<commit_message>
Align the test report and the presentation script with proposal v1.1
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ACBI-TSR-2026-10-13-01</t>
+          <t>ACBI-TSR-2026-10-14-01</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ACBI, commit 177b4cf</t>
+          <t>ACBI, commit 2194ad7</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1919,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>• ACBI_Technical_Solution_Proposal_v1.0.docx (đề xuất giải pháp)</t>
+          <t>• ACBI_Technical_Solution_Proposal_v1.1.docx (đề xuất giải pháp, bản đã cập nhật theo hệ thống đã xây)</t>
         </is>
       </c>
     </row>
@@ -7798,7 +7798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7854,81 +7854,81 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi (tối đa 1000 ký tự); ngày dữ liệu; danh mục chỉ số, chiều và tên khu vực, nhà máy đã duyệt; phiếu yêu cầu của lượt trước; tối đa 6 lượt gần nhất gồm câu hỏi và câu trả lời, trong đó số tiền, tỷ lệ và số thập phân đã thay bằng [số] (từ commit 68c9ade).</t>
+          <t>Câu hỏi (tối đa 1000 ký tự); ngày dữ liệu; toàn bộ danh mục chỉ số đã duyệt (không lọc theo vai trò), chiều và thành viên (tối đa 40 mỗi chiều, kèm mã nhà máy); phiếu yêu cầu và câu hỏi làm rõ đang chờ của lượt trước; tối đa 6 lượt gần nhất gồm câu hỏi và câu trả lời, trong đó số tiền có dấu phân cách hàng nghìn và tỷ lệ có phần thập phân đã thay bằng [số]. Số nguyên không định dạng (ví dụ 5%) không bị thay.</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Dòng kết quả; số tiền và tỷ lệ của câu trả lời trước; mật khẩu, khóa, vai trò, mã người dùng</t>
+          <t>Dòng kết quả; mật khẩu, khóa, vai trò, mã người dùng</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Luôn dùng khi câu cần AI hiểu (câu rõ ràng được tra từ điển, không gọi AI)</t>
+          <t>Dùng cho câu mà quy tắc của backend không đọc được. Đọc câu rõ ràng bằng quy tắc (LOCAL_INTENT_ENABLED) là tùy chọn, mặc định tắt trong Docker Compose; cũng là phương án dự phòng khi AI bận</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Dùng (Gemini, LiteRouter)</t>
+          <t>Dùng (Gemini, LiteRouter); LOCAL_INTENT_ENABLED bật</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Đề xuất SQL (sql_candidate)</t>
+          <t>Hỏi đáp về dữ liệu và câu trả lời trước (converse)</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Câu ngoài mẫu: AI đề xuất câu SELECT</t>
+          <t>Trả lời câu hỏi về chính dữ liệu (có những chỉ số nào, định nghĩa, phạm vi ngày) hoặc về câu trả lời vừa rồi</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi; phiếu yêu cầu (không có kỳ, nhà máy, khu vực với chỉ số doanh thu, sản lượng, tỷ lệ lỗi); định nghĩa chỉ số đã duyệt; ánh xạ nguồn và quy tắc nối bảng; tên bảng và cột được phép theo vai trò; tối đa 2 SQL mẫu đã duyệt; lý do khi cần sửa.</t>
+          <t>Câu hỏi; metadata theo vai trò (chỉ số, chiều và thành viên, ngày phủ dữ liệu, tên bảng và cột được phép); mô tả câu trả lời trước gồm cả văn bản trả lời kèm số liệu (không che số).</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Dòng kết quả; toàn bộ lược đồ không giới hạn; khóa, mật khẩu, mã người dùng</t>
+          <t>Bảng kết quả (các dòng); khóa, mật khẩu, mã người dùng</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>EXTERNAL_METADATA_ENABLED (mặc định tắt trong Docker Compose; chủ dự án duyệt ngày 20/09/2026)</t>
+          <t>Không có công tắc riêng; dùng khi AI được bật</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Bật</t>
+          <t>Dùng</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Chọn biểu đồ (visualize)</t>
+          <t>Đề xuất SQL (sql_candidate)</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Chọn loại biểu đồ khi quy tắc không quyết được</t>
+          <t>Câu ngoài mẫu: AI đề xuất câu SELECT</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi; mô tả kết quả: số dòng, tên cột, kiểu cột (số, thời gian, nhóm), có thứ tự hay không.</t>
+          <t>Câu hỏi; phiếu yêu cầu (không có kỳ, nhà máy, khu vực với chỉ số doanh thu, sản lượng, tỷ lệ lỗi; chỉ số tăng trưởng giữ các trường này); định nghĩa chỉ số đã duyệt; ánh xạ nguồn và quy tắc nối bảng (tăng trưởng còn kèm SQL tham chiếu); tên bảng và cột được phép theo vai trò; tối đa 2 SQL mẫu đã duyệt; lý do khi cần sửa.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Giá trị trong các dòng kết quả</t>
+          <t>Dòng kết quả; toàn bộ lược đồ không giới hạn; khóa, mật khẩu, mã người dùng</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>EXTERNAL_METADATA_ENABLED</t>
+          <t>EXTERNAL_METADATA_ENABLED (mặc định tắt trong Docker Compose; chủ dự án duyệt ngày 20/09/2026). Khi tắt, chỉ đường mẫu chạy</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -7940,125 +7940,141 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Tóm tắt bằng AI (summarize)</t>
+          <t>Chọn biểu đồ (visualize)</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Viết câu tóm tắt từ dòng kết quả</t>
+          <t>Chọn loại biểu đồ khi quy tắc không quyết được</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Các dòng kết quả (nếu bật).</t>
+          <t>Câu hỏi; mô tả kết quả: số dòng, tên cột, kiểu cột (số, thời gian, nhóm), có thứ tự hay không, số giá trị khác nhau, có đủ dữ liệu hay không. Chỉ gửi khi quy tắc của backend (một giá trị là thẻ, trục ngày là đường, hai nhóm là cột chồng, một tổng nhỏ là tròn) không chọn được biểu đồ.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Giá trị trong các dòng kết quả</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>SEND_RESULTS_TO_LLM và EXTERNAL_RESULTS_ENABLED (mặc định tắt); câu tóm tắt mặc định do backend tự dựng</t>
+          <t>EXTERNAL_METADATA_ENABLED; khi tắt, kết quả luôn hiển thị dạng bảng</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Tắt</t>
+          <t>Bật</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>Tóm tắt bằng AI (summarize)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Viết câu tóm tắt từ dòng kết quả</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Các dòng kết quả (nếu bật).</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>SEND_RESULTS_TO_LLM và EXTERNAL_RESULTS_ENABLED (mặc định tắt); câu tóm tắt mặc định do backend tự dựng</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Tắt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
           <t>Chuyển giọng nói</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Chuyển file ghi âm thành văn bản</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>File ghi âm khi người dùng bấm ghi âm và dừng.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Cần khóa Groq; người dùng tự bấm ghi âm</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Chưa bật (không có khóa Groq trên Vercel)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Nhà cung cấp AI đang dùng: Gemini và LiteRouter (bản demo), Groq tùy chọn, Ollama chạy trên máy nội bộ (không ra ngoài).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Chưa có: rà soát điều khoản lưu giữ và huấn luyện dữ liệu của từng nhà cung cấp, đặc biệt gói miễn phí; bảng phân loại dữ liệu theo mức nhạy cảm; che (mask) thêm các trường nhạy cảm nếu dùng dữ liệu thật. Đây là điều kiện trước khi thí điểm với dữ liệu thật.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Kho dữ liệu: backend truy cập bằng tài khoản chỉ đọc, AI không có đường nào tới kho dữ liệu.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Cách đọc các cột</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Lời gọi AI</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>Một loại yêu cầu mà backend gửi cho dịch vụ AI bên ngoài.</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Nội dung được gửi / Không gửi</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>Dữ liệu rời khỏi hệ thống trong lời gọi đó, và dữ liệu không bao giờ gửi (ví dụ dòng kết quả, mật khẩu, khóa).</t>
         </is>
       </c>
       <c r="C20" s="23" t="n"/>
@@ -8066,15 +8082,15 @@
       <c r="E20" s="23" t="n"/>
       <c r="F20" s="23" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>Công tắc điều khiển</t>
+          <t>Nội dung được gửi / Không gửi</t>
         </is>
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>Biến cấu hình bật hoặc tắt việc gửi; mặc định thường là tắt.</t>
+          <t>Dữ liệu rời khỏi hệ thống trong lời gọi đó, và dữ liệu không bao giờ gửi (ví dụ dòng kết quả, mật khẩu, khóa).</t>
         </is>
       </c>
       <c r="C21" s="23" t="n"/>
@@ -8082,15 +8098,15 @@
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n"/>
     </row>
-    <row r="22" ht="32" customHeight="1">
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Trạng thái trên bản demo</t>
+          <t>Công tắc điều khiển</t>
         </is>
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>Lời gọi này đang dùng hay không trên bản demo hiện tại.</t>
+          <t>Biến cấu hình bật hoặc tắt việc gửi; mặc định thường là tắt.</t>
         </is>
       </c>
       <c r="C22" s="23" t="n"/>
@@ -8098,15 +8114,31 @@
       <c r="E22" s="23" t="n"/>
       <c r="F22" s="23" t="n"/>
     </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Trạng thái trên bản demo</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Lời gọi này đang dùng hay không trên bản demo hiện tại.</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B21:F21"/>
-    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8463,7 +8495,7 @@
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="43" t="inlineStr">
         <is>
-          <t>Ghi chú: token đo bằng Ollama (qwen2.5:7b) trên đúng lời nhắc của hệ thống. Cột D lấy từ bộ 161 ca kiểm thử: trung bình 0,47 lời gọi mỗi câu, 67% câu không cần AI (câu rõ ràng tra từ điển); phân bổ giữa 3 loại lời gọi là ước lượng. Cột E: mọi câu cần AI hiểu và AI viết SQL.</t>
+          <t>Ghi chú: token đo bằng Ollama (qwen2.5:7b) trên đúng lời nhắc của hệ thống. Cột D lấy từ bộ 161 ca kiểm thử: trung bình 0,47 lời gọi mỗi câu, 67% câu không cần AI vì bản demo bật LOCAL_INTENT_ENABLED (đọc câu rõ ràng bằng quy tắc); tùy chọn này mặc định tắt, khi tắt mọi câu dữ liệu cần AI hiểu nên chi phí gần cột E; phân bổ giữa 3 loại lời gọi là ước lượng. Cột E: mọi câu cần AI hiểu và AI viết SQL. Chưa tính lần sửa SQL, tóm tắt và trả lời về dữ liệu.</t>
         </is>
       </c>
       <c r="B24" s="17" t="n"/>
@@ -9052,6 +9084,22 @@
       <c r="B59" s="47">
         <f>D47*$B$5</f>
         <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Số câu mỗi tháng để API Haiku 5.5 (kịch bản xấu) bằng GPU 500 USD/tháng (cận trên)</t>
+        </is>
+      </c>
+      <c r="B60" s="47">
+        <f>500/(D27/1000)</f>
+        <v/>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Khoảng hòa vốn là từ B56 (GPU rẻ nhất) đến B60 (GPU 500 USD).</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -9442,7 +9490,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>nhánh main, commit 177b4cf</t>
+          <t>nhánh main, commit 2194ad7</t>
         </is>
       </c>
     </row>
@@ -9538,7 +9586,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -9747,7 +9795,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -9816,7 +9864,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -9885,7 +9933,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -9955,7 +10003,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -10025,7 +10073,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -10095,7 +10143,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -10165,7 +10213,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -10235,7 +10283,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -10304,7 +10352,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -10374,7 +10422,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -10442,7 +10490,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -10509,7 +10557,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -10576,7 +10624,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -10643,7 +10691,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -10711,7 +10759,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -10780,7 +10828,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -10850,7 +10898,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -10920,7 +10968,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -10990,7 +11038,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -11060,7 +11108,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -11129,7 +11177,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -11198,7 +11246,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -11267,7 +11315,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -11336,7 +11384,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -11796,7 +11844,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -11863,7 +11911,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -11930,7 +11978,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -11997,7 +12045,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -12064,7 +12112,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -12131,7 +12179,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -12198,7 +12246,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -12265,7 +12313,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -12332,7 +12380,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -12399,7 +12447,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -12467,7 +12515,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -12535,7 +12583,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -12607,7 +12655,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -12675,7 +12723,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -12742,7 +12790,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -12810,7 +12858,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -12879,7 +12927,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -12946,7 +12994,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -13013,7 +13061,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -13080,7 +13128,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -13147,7 +13195,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -13214,7 +13262,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -13281,7 +13329,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -13348,7 +13396,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -13415,7 +13463,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -13482,7 +13530,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -13550,7 +13598,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -13618,7 +13666,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -13685,7 +13733,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -13752,7 +13800,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -13819,7 +13867,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -13887,7 +13935,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -13968,7 +14016,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -14039,7 +14087,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -14108,7 +14156,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -14177,7 +14225,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -14246,7 +14294,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -14315,7 +14363,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -14383,7 +14431,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -14450,7 +14498,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -14517,7 +14565,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -14584,7 +14632,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -14651,7 +14699,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -14719,7 +14767,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -14788,7 +14836,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -14856,7 +14904,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -14924,7 +14972,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -14992,7 +15040,7 @@
       </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr">
@@ -15059,7 +15107,7 @@
       </c>
       <c r="L50" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M50" s="8" t="inlineStr">
@@ -15126,7 +15174,7 @@
       </c>
       <c r="L51" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M51" s="8" t="inlineStr">
@@ -15194,7 +15242,7 @@
       </c>
       <c r="L52" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M52" s="8" t="inlineStr">
@@ -15262,7 +15310,7 @@
       </c>
       <c r="L53" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M53" s="8" t="inlineStr">
@@ -15330,7 +15378,7 @@
       </c>
       <c r="L54" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M54" s="8" t="inlineStr">
@@ -15411,7 +15459,7 @@
       </c>
       <c r="L55" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M55" s="8" t="inlineStr">
@@ -15492,7 +15540,7 @@
       </c>
       <c r="L56" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M56" s="8" t="inlineStr">
@@ -15572,7 +15620,7 @@
       </c>
       <c r="L57" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M57" s="8" t="inlineStr">
@@ -15643,7 +15691,7 @@
       </c>
       <c r="L58" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M58" s="8" t="inlineStr">
@@ -15711,7 +15759,7 @@
       </c>
       <c r="L59" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M59" s="8" t="inlineStr">
@@ -15779,7 +15827,7 @@
       </c>
       <c r="L60" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M60" s="8" t="inlineStr">
@@ -15868,7 +15916,7 @@
       </c>
       <c r="L61" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M61" s="8" t="inlineStr">
@@ -15948,7 +15996,7 @@
       </c>
       <c r="L62" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M62" s="8" t="inlineStr">
@@ -16027,7 +16075,7 @@
       </c>
       <c r="L63" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M63" s="8" t="inlineStr">
@@ -16099,7 +16147,7 @@
       </c>
       <c r="L64" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M64" s="8" t="inlineStr">
@@ -16171,7 +16219,7 @@
       </c>
       <c r="L65" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M65" s="8" t="inlineStr">
@@ -16256,7 +16304,7 @@
       </c>
       <c r="L66" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M66" s="8" t="inlineStr">
@@ -16343,7 +16391,7 @@
       </c>
       <c r="L67" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M67" s="8" t="inlineStr">
@@ -16418,7 +16466,7 @@
       </c>
       <c r="L68" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M68" s="8" t="inlineStr">
@@ -16487,7 +16535,7 @@
       </c>
       <c r="L69" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M69" s="8" t="inlineStr">
@@ -16555,7 +16603,7 @@
       </c>
       <c r="L70" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M70" s="8" t="inlineStr">
@@ -16627,7 +16675,7 @@
       </c>
       <c r="L71" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M71" s="8" t="inlineStr">
@@ -16696,7 +16744,7 @@
       </c>
       <c r="L72" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M72" s="8" t="inlineStr">
@@ -16765,7 +16813,7 @@
       </c>
       <c r="L73" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M73" s="8" t="inlineStr">
@@ -16838,7 +16886,7 @@
       </c>
       <c r="L74" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M74" s="8" t="inlineStr">
@@ -16907,7 +16955,7 @@
       </c>
       <c r="L75" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M75" s="8" t="inlineStr">
@@ -16976,7 +17024,7 @@
       </c>
       <c r="L76" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M76" s="8" t="inlineStr">
@@ -17045,7 +17093,7 @@
       </c>
       <c r="L77" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M77" s="8" t="inlineStr">
@@ -17114,7 +17162,7 @@
       </c>
       <c r="L78" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M78" s="8" t="inlineStr">
@@ -17183,7 +17231,7 @@
       </c>
       <c r="L79" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M79" s="8" t="inlineStr">
@@ -17252,7 +17300,7 @@
       </c>
       <c r="L80" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M80" s="8" t="inlineStr">
@@ -17322,7 +17370,7 @@
       </c>
       <c r="L81" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M81" s="8" t="inlineStr">
@@ -17390,7 +17438,7 @@
       </c>
       <c r="L82" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M82" s="8" t="inlineStr">
@@ -17458,7 +17506,7 @@
       </c>
       <c r="L83" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M83" s="8" t="inlineStr">
@@ -17527,7 +17575,7 @@
       </c>
       <c r="L84" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M84" s="8" t="inlineStr">
@@ -17595,7 +17643,7 @@
       </c>
       <c r="L85" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M85" s="8" t="inlineStr">
@@ -17665,7 +17713,7 @@
       </c>
       <c r="L86" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M86" s="8" t="inlineStr">
@@ -17734,7 +17782,7 @@
       </c>
       <c r="L87" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M87" s="8" t="inlineStr">
@@ -17804,7 +17852,7 @@
       </c>
       <c r="L88" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M88" s="8" t="inlineStr">
@@ -17871,7 +17919,7 @@
       </c>
       <c r="L89" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M89" s="8" t="inlineStr">
@@ -17938,7 +17986,7 @@
       </c>
       <c r="L90" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M90" s="8" t="inlineStr">
@@ -18007,7 +18055,7 @@
       </c>
       <c r="L91" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M91" s="8" t="inlineStr">
@@ -18468,7 +18516,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -18537,7 +18585,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -18605,7 +18653,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -18675,7 +18723,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -18745,7 +18793,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -18815,7 +18863,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -18882,7 +18930,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -18949,7 +18997,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -19016,7 +19064,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -19083,7 +19131,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -19150,7 +19198,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -19217,7 +19265,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -19288,7 +19336,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -19355,7 +19403,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -19422,7 +19470,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -19489,7 +19537,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -19557,7 +19605,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -19627,7 +19675,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -19697,7 +19745,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -19774,7 +19822,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -19844,7 +19892,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -19913,7 +19961,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -19980,7 +20028,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -20047,7 +20095,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -20114,7 +20162,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -20181,7 +20229,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -20248,7 +20296,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -20315,7 +20363,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -20382,7 +20430,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -20453,7 +20501,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -20520,7 +20568,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -20590,7 +20638,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -20659,7 +20707,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -20728,7 +20776,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -20798,7 +20846,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -20870,7 +20918,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -20939,7 +20987,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -21009,7 +21057,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -21078,7 +21126,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -21154,7 +21202,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -21224,7 +21272,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -21292,7 +21340,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -21361,7 +21409,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -21433,7 +21481,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -21503,7 +21551,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -21572,7 +21620,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -21646,7 +21694,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -22109,7 +22157,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -22178,7 +22226,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -22247,7 +22295,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -22316,7 +22364,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -22385,7 +22433,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -22454,7 +22502,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -22523,7 +22571,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -22592,7 +22640,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -22661,7 +22709,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -22730,7 +22778,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -22799,7 +22847,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -22868,7 +22916,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -22937,7 +22985,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -23006,7 +23054,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -23075,7 +23123,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -23144,7 +23192,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -23213,7 +23261,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -23282,7 +23330,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -23351,7 +23399,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -23420,7 +23468,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -23489,7 +23537,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -23558,7 +23606,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -23627,7 +23675,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -23696,7 +23744,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -23765,7 +23813,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -23834,7 +23882,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -23903,7 +23951,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -23972,7 +24020,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -24041,7 +24089,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -24110,7 +24158,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -24179,7 +24227,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -24248,7 +24296,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -24317,7 +24365,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -24386,7 +24434,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -24455,7 +24503,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -24524,7 +24572,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -24593,7 +24641,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -24662,7 +24710,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -24731,7 +24779,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -24800,7 +24848,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -24869,7 +24917,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -24938,7 +24986,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -25007,7 +25055,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -25076,7 +25124,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -25145,7 +25193,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -25214,7 +25262,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -25283,7 +25331,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -25352,7 +25400,7 @@
       </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Excel data-sent sheet: no factory-specific wording
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ACBI, commit 2194ad7</t>
+          <t>ACBI, commit 08985c9</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi (tối đa 1000 ký tự); ngày dữ liệu; toàn bộ danh mục chỉ số đã duyệt (không lọc theo vai trò), chiều và thành viên (tối đa 40 mỗi chiều, kèm mã nhà máy); phiếu yêu cầu và câu hỏi làm rõ đang chờ của lượt trước; tối đa 6 lượt gần nhất gồm câu hỏi và câu trả lời, trong đó số tiền có dấu phân cách hàng nghìn và tỷ lệ có phần thập phân đã thay bằng [số]. Số nguyên không định dạng (ví dụ 5%) không bị thay.</t>
+          <t>Câu hỏi (tối đa 1000 ký tự); ngày dữ liệu; toàn bộ danh mục chỉ số đã duyệt (không lọc theo vai trò), chiều và thành viên (tối đa 40 mỗi chiều, kèm mã định danh); phiếu yêu cầu và câu hỏi làm rõ đang chờ của lượt trước; tối đa 6 lượt gần nhất gồm câu hỏi và câu trả lời, trong đó số tiền có dấu phân cách hàng nghìn và tỷ lệ có phần thập phân đã thay bằng [số]. Số nguyên không định dạng (ví dụ 5%) không bị thay.</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Câu hỏi; phiếu yêu cầu (không có kỳ, nhà máy, khu vực với chỉ số doanh thu, sản lượng, tỷ lệ lỗi; chỉ số tăng trưởng giữ các trường này); định nghĩa chỉ số đã duyệt; ánh xạ nguồn và quy tắc nối bảng (tăng trưởng còn kèm SQL tham chiếu); tên bảng và cột được phép theo vai trò; tối đa 2 SQL mẫu đã duyệt; lý do khi cần sửa.</t>
+          <t>Câu hỏi; phiếu yêu cầu (không có kỳ và các bộ lọc theo chiều với chỉ số doanh thu, sản lượng, tỷ lệ lỗi; chỉ số tăng trưởng giữ các trường này); định nghĩa chỉ số đã duyệt; ánh xạ nguồn và quy tắc nối bảng (tăng trưởng còn kèm SQL tham chiếu); tên bảng và cột được phép theo vai trò; tối đa 2 SQL mẫu đã duyệt; lý do khi cần sửa.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>nhánh main, commit 2194ad7</t>
+          <t>nhánh main, commit 08985c9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix review findings: first-run figures, tested commit and date, over-absolute claims
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ACBI-TSR-2026-10-14-01</t>
+          <t>ACBI-TSR-2026-10-13-01</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ACBI, commit 08985c9</t>
+          <t>ACBI, commit 177b4cf</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -9490,7 +9490,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>nhánh main, commit 08985c9</t>
+          <t>nhánh main, commit 177b4cf</t>
         </is>
       </c>
     </row>
@@ -9586,7 +9586,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -9795,7 +9795,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -9933,7 +9933,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -10073,7 +10073,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -10213,7 +10213,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -10352,7 +10352,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -10490,7 +10490,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -10557,7 +10557,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -10624,7 +10624,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -10691,7 +10691,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -10828,7 +10828,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -11108,7 +11108,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -11384,7 +11384,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -11844,7 +11844,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -11911,7 +11911,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -11978,7 +11978,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -12045,7 +12045,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -12112,7 +12112,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -12179,7 +12179,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -12583,7 +12583,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -12655,7 +12655,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -12723,7 +12723,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -12790,7 +12790,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -12858,7 +12858,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -12927,7 +12927,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -13061,7 +13061,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -13195,7 +13195,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -13262,7 +13262,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -13463,7 +13463,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -13935,7 +13935,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -14016,7 +14016,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -14087,7 +14087,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -14156,7 +14156,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -14225,7 +14225,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -14431,7 +14431,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -14498,7 +14498,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -14565,7 +14565,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -14632,7 +14632,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -14767,7 +14767,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -14836,7 +14836,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -14904,7 +14904,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -15040,7 +15040,7 @@
       </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="L50" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M50" s="8" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="L51" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M51" s="8" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="L52" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M52" s="8" t="inlineStr">
@@ -15310,7 +15310,7 @@
       </c>
       <c r="L53" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M53" s="8" t="inlineStr">
@@ -15378,7 +15378,7 @@
       </c>
       <c r="L54" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M54" s="8" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="L55" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M55" s="8" t="inlineStr">
@@ -15540,7 +15540,7 @@
       </c>
       <c r="L56" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M56" s="8" t="inlineStr">
@@ -15620,7 +15620,7 @@
       </c>
       <c r="L57" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M57" s="8" t="inlineStr">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="L58" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M58" s="8" t="inlineStr">
@@ -15759,7 +15759,7 @@
       </c>
       <c r="L59" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M59" s="8" t="inlineStr">
@@ -15827,7 +15827,7 @@
       </c>
       <c r="L60" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M60" s="8" t="inlineStr">
@@ -15916,7 +15916,7 @@
       </c>
       <c r="L61" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M61" s="8" t="inlineStr">
@@ -15996,7 +15996,7 @@
       </c>
       <c r="L62" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M62" s="8" t="inlineStr">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="L63" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M63" s="8" t="inlineStr">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="L64" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M64" s="8" t="inlineStr">
@@ -16219,7 +16219,7 @@
       </c>
       <c r="L65" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M65" s="8" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="L66" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M66" s="8" t="inlineStr">
@@ -16391,7 +16391,7 @@
       </c>
       <c r="L67" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M67" s="8" t="inlineStr">
@@ -16466,7 +16466,7 @@
       </c>
       <c r="L68" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M68" s="8" t="inlineStr">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="L69" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M69" s="8" t="inlineStr">
@@ -16603,7 +16603,7 @@
       </c>
       <c r="L70" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M70" s="8" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="L71" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M71" s="8" t="inlineStr">
@@ -16744,7 +16744,7 @@
       </c>
       <c r="L72" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M72" s="8" t="inlineStr">
@@ -16813,7 +16813,7 @@
       </c>
       <c r="L73" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M73" s="8" t="inlineStr">
@@ -16886,7 +16886,7 @@
       </c>
       <c r="L74" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M74" s="8" t="inlineStr">
@@ -16955,7 +16955,7 @@
       </c>
       <c r="L75" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M75" s="8" t="inlineStr">
@@ -17024,7 +17024,7 @@
       </c>
       <c r="L76" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M76" s="8" t="inlineStr">
@@ -17093,7 +17093,7 @@
       </c>
       <c r="L77" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M77" s="8" t="inlineStr">
@@ -17162,7 +17162,7 @@
       </c>
       <c r="L78" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M78" s="8" t="inlineStr">
@@ -17231,7 +17231,7 @@
       </c>
       <c r="L79" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M79" s="8" t="inlineStr">
@@ -17300,7 +17300,7 @@
       </c>
       <c r="L80" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M80" s="8" t="inlineStr">
@@ -17370,7 +17370,7 @@
       </c>
       <c r="L81" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M81" s="8" t="inlineStr">
@@ -17438,7 +17438,7 @@
       </c>
       <c r="L82" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M82" s="8" t="inlineStr">
@@ -17506,7 +17506,7 @@
       </c>
       <c r="L83" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M83" s="8" t="inlineStr">
@@ -17575,7 +17575,7 @@
       </c>
       <c r="L84" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M84" s="8" t="inlineStr">
@@ -17643,7 +17643,7 @@
       </c>
       <c r="L85" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M85" s="8" t="inlineStr">
@@ -17713,7 +17713,7 @@
       </c>
       <c r="L86" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M86" s="8" t="inlineStr">
@@ -17782,7 +17782,7 @@
       </c>
       <c r="L87" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M87" s="8" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="L88" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M88" s="8" t="inlineStr">
@@ -17919,7 +17919,7 @@
       </c>
       <c r="L89" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M89" s="8" t="inlineStr">
@@ -17986,7 +17986,7 @@
       </c>
       <c r="L90" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M90" s="8" t="inlineStr">
@@ -18055,7 +18055,7 @@
       </c>
       <c r="L91" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M91" s="8" t="inlineStr">
@@ -18516,7 +18516,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -18585,7 +18585,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -18653,7 +18653,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -18723,7 +18723,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -18793,7 +18793,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -18930,7 +18930,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -18997,7 +18997,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -19064,7 +19064,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -19131,7 +19131,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -19198,7 +19198,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -19265,7 +19265,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -19336,7 +19336,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -19470,7 +19470,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -19537,7 +19537,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -19675,7 +19675,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -19745,7 +19745,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -19822,7 +19822,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -19892,7 +19892,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -19961,7 +19961,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -20095,7 +20095,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -20162,7 +20162,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -20229,7 +20229,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -20296,7 +20296,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -20363,7 +20363,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -20430,7 +20430,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -20568,7 +20568,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -20638,7 +20638,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -20707,7 +20707,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -20776,7 +20776,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -20846,7 +20846,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -20918,7 +20918,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -20987,7 +20987,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -21126,7 +21126,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -21202,7 +21202,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -21272,7 +21272,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -21340,7 +21340,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -21409,7 +21409,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -21481,7 +21481,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -21551,7 +21551,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -21620,7 +21620,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -21694,7 +21694,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -22157,7 +22157,7 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -22226,7 +22226,7 @@
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
@@ -22295,7 +22295,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -22364,7 +22364,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -22433,7 +22433,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -22502,7 +22502,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -22571,7 +22571,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -22640,7 +22640,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -22709,7 +22709,7 @@
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -22778,7 +22778,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -22847,7 +22847,7 @@
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -22916,7 +22916,7 @@
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -23054,7 +23054,7 @@
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -23123,7 +23123,7 @@
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -23192,7 +23192,7 @@
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -23261,7 +23261,7 @@
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -23330,7 +23330,7 @@
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
@@ -23399,7 +23399,7 @@
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -23468,7 +23468,7 @@
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -23537,7 +23537,7 @@
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -23606,7 +23606,7 @@
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -23675,7 +23675,7 @@
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -23744,7 +23744,7 @@
       </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -23882,7 +23882,7 @@
       </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M27" s="8" t="inlineStr">
@@ -23951,7 +23951,7 @@
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -24020,7 +24020,7 @@
       </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -24089,7 +24089,7 @@
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -24158,7 +24158,7 @@
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
@@ -24227,7 +24227,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -24296,7 +24296,7 @@
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -24365,7 +24365,7 @@
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -24434,7 +24434,7 @@
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
@@ -24503,7 +24503,7 @@
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -24572,7 +24572,7 @@
       </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M37" s="8" t="inlineStr">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -24710,7 +24710,7 @@
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
@@ -24779,7 +24779,7 @@
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -24848,7 +24848,7 @@
       </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
@@ -24917,7 +24917,7 @@
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -24986,7 +24986,7 @@
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -25055,7 +25055,7 @@
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -25124,7 +25124,7 @@
       </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
@@ -25193,7 +25193,7 @@
       </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
@@ -25262,7 +25262,7 @@
       </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
@@ -25331,7 +25331,7 @@
       </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
@@ -25400,7 +25400,7 @@
       </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M49" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Drop the staff-cost placeholders from the Excel, the proposal and the script
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -10981,12 +10981,12 @@
       </c>
       <c r="D52" s="38" t="inlineStr">
         <is>
-          <t>[điền]</t>
+          <t>Ngoài phạm vi ước tính</t>
         </is>
       </c>
       <c r="F52" s="14" t="inlineStr">
         <is>
-          <t>Chưa ước tính. Đây là khoản lớn thường bị bỏ sót khi tự vận hành mô hình.</t>
+          <t>Không nằm trong ước tính này. Đây là khoản lớn thường bị bỏ sót khi tự vận hành mô hình.</t>
         </is>
       </c>
     </row>
@@ -11244,7 +11244,7 @@
     <row r="72" ht="52" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>Việc cần làm trước khi chốt: (1) thêm nhà cung cấp Claude và chạy bộ 161 ca; (2) đo token bằng count_tokens; (3) xác nhận điều khoản dữ liệu của nhà cung cấp; (4) điền chi phí nhân sự.</t>
+          <t>Việc cần làm trước khi chốt: (1) thêm nhà cung cấp Claude và chạy bộ 161 ca; (2) đo token bằng count_tokens; (3) xác nhận điều khoản dữ liệu của nhà cung cấp; (4) ước tính chi phí nhân sự.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set the document author to the account name instead of the generator library
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -418,6 +418,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -443,6 +446,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -468,6 +474,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -493,6 +502,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -518,6 +530,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -543,6 +558,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -568,6 +586,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -593,6 +614,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -618,6 +642,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -643,6 +670,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -668,6 +698,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -693,6 +726,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -718,6 +754,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -743,6 +782,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -768,6 +810,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -793,6 +838,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -818,6 +866,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -843,6 +894,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -868,6 +922,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -893,6 +950,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -918,6 +978,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -943,6 +1006,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -968,6 +1034,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -993,6 +1062,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1974,13 +2046,13 @@
           <t>Số ca kiểm thử trong bộ đó. Một ca là một câu hỏi (hoặc một chuỗi câu hỏi nối tiếp) cùng điều kiện đạt.</t>
         </is>
       </c>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="23" t="n"/>
-      <c r="E49" s="23" t="n"/>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="23" t="n"/>
-      <c r="H49" s="23" t="n"/>
-      <c r="I49" s="23" t="n"/>
+      <c r="C49" s="17" t="n"/>
+      <c r="D49" s="17" t="n"/>
+      <c r="E49" s="17" t="n"/>
+      <c r="F49" s="17" t="n"/>
+      <c r="G49" s="17" t="n"/>
+      <c r="H49" s="17" t="n"/>
+      <c r="I49" s="18" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="21" t="inlineStr">
@@ -1993,13 +2065,13 @@
           <t>Số ca đạt mọi yêu cầu.</t>
         </is>
       </c>
-      <c r="C50" s="23" t="n"/>
-      <c r="D50" s="23" t="n"/>
-      <c r="E50" s="23" t="n"/>
-      <c r="F50" s="23" t="n"/>
-      <c r="G50" s="23" t="n"/>
-      <c r="H50" s="23" t="n"/>
-      <c r="I50" s="23" t="n"/>
+      <c r="C50" s="17" t="n"/>
+      <c r="D50" s="17" t="n"/>
+      <c r="E50" s="17" t="n"/>
+      <c r="F50" s="17" t="n"/>
+      <c r="G50" s="17" t="n"/>
+      <c r="H50" s="17" t="n"/>
+      <c r="I50" s="18" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="21" t="inlineStr">
@@ -2012,13 +2084,13 @@
           <t>Số ca sai ít nhất một yêu cầu (sai số, sai quyền, trả lời khi lẽ ra phải hỏi lại...).</t>
         </is>
       </c>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="23" t="n"/>
-      <c r="E51" s="23" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="23" t="n"/>
-      <c r="H51" s="23" t="n"/>
-      <c r="I51" s="23" t="n"/>
+      <c r="C51" s="17" t="n"/>
+      <c r="D51" s="17" t="n"/>
+      <c r="E51" s="17" t="n"/>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="17" t="n"/>
+      <c r="H51" s="17" t="n"/>
+      <c r="I51" s="18" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="21" t="inlineStr">
@@ -2031,13 +2103,13 @@
           <t>Số ca không đánh giá được vì dịch vụ AI báo bận. Con số này nói về hạn mức dịch vụ AI, không nói về độ đúng của hệ thống.</t>
         </is>
       </c>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="23" t="n"/>
-      <c r="E52" s="23" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="23" t="n"/>
-      <c r="I52" s="23" t="n"/>
+      <c r="C52" s="17" t="n"/>
+      <c r="D52" s="17" t="n"/>
+      <c r="E52" s="17" t="n"/>
+      <c r="F52" s="17" t="n"/>
+      <c r="G52" s="17" t="n"/>
+      <c r="H52" s="17" t="n"/>
+      <c r="I52" s="18" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="21" t="inlineStr">
@@ -2050,13 +2122,13 @@
           <t>Số ca chưa chạy: bằng Tổng số ca trừ Passed, Failed, Blocked.</t>
         </is>
       </c>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="23" t="n"/>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
+      <c r="C53" s="17" t="n"/>
+      <c r="D53" s="17" t="n"/>
+      <c r="E53" s="17" t="n"/>
+      <c r="F53" s="17" t="n"/>
+      <c r="G53" s="17" t="n"/>
+      <c r="H53" s="17" t="n"/>
+      <c r="I53" s="18" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="21" t="inlineStr">
@@ -2069,13 +2141,13 @@
           <t>Passed cộng Failed: số ca đã thật sự cho ra kết luận đúng hoặc sai.</t>
         </is>
       </c>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="23" t="n"/>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
+      <c r="C54" s="17" t="n"/>
+      <c r="D54" s="17" t="n"/>
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="17" t="n"/>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="18" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="21" t="inlineStr">
@@ -2088,13 +2160,13 @@
           <t>Passed chia cho Đã thực thi. Ví dụ 100% nghĩa là mọi ca đã chạy đều đạt.</t>
         </is>
       </c>
-      <c r="C55" s="23" t="n"/>
-      <c r="D55" s="23" t="n"/>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="23" t="n"/>
-      <c r="H55" s="23" t="n"/>
-      <c r="I55" s="23" t="n"/>
+      <c r="C55" s="17" t="n"/>
+      <c r="D55" s="17" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="17" t="n"/>
+      <c r="G55" s="17" t="n"/>
+      <c r="H55" s="17" t="n"/>
+      <c r="I55" s="18" t="n"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="21" t="inlineStr">
@@ -2107,13 +2179,13 @@
           <t>Kết quả trước khi chạy lại các ca báo AI bận: cho biết hạn mức AI ảnh hưởng đến lần chạy đầu bao nhiêu.</t>
         </is>
       </c>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="23" t="n"/>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="23" t="n"/>
-      <c r="H56" s="23" t="n"/>
-      <c r="I56" s="23" t="n"/>
+      <c r="C56" s="17" t="n"/>
+      <c r="D56" s="17" t="n"/>
+      <c r="E56" s="17" t="n"/>
+      <c r="F56" s="17" t="n"/>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="18" t="n"/>
     </row>
     <row r="57" ht="32" customHeight="1">
       <c r="A57" s="21" t="inlineStr">
@@ -2126,13 +2198,13 @@
           <t>Mục tiêu đặt ra trước, thực tế đo được, và kết luận Đạt hoặc Chưa đạt. Hiệu năng Chưa đạt nghĩa là đo tải 5 người cùng lúc chưa đủ 95% yêu cầu hoàn tất dưới 15 giây.</t>
         </is>
       </c>
-      <c r="C57" s="23" t="n"/>
-      <c r="D57" s="23" t="n"/>
-      <c r="E57" s="23" t="n"/>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="23" t="n"/>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="n"/>
+      <c r="C57" s="17" t="n"/>
+      <c r="D57" s="17" t="n"/>
+      <c r="E57" s="17" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="18" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -2195,11 +2267,11 @@
           <t>Số liệu bằng kho dữ liệu</t>
         </is>
       </c>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="25" t="n"/>
-      <c r="G62" s="25" t="n"/>
-      <c r="H62" s="25" t="n"/>
-      <c r="I62" s="25" t="n"/>
+      <c r="E62" s="17" t="n"/>
+      <c r="F62" s="17" t="n"/>
+      <c r="G62" s="17" t="n"/>
+      <c r="H62" s="17" t="n"/>
+      <c r="I62" s="18" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="25" t="inlineStr">
@@ -2220,11 +2292,11 @@
           <t>Phải bằng 0 để các ca Passed</t>
         </is>
       </c>
-      <c r="E63" s="25" t="n"/>
-      <c r="F63" s="25" t="n"/>
-      <c r="G63" s="25" t="n"/>
-      <c r="H63" s="25" t="n"/>
-      <c r="I63" s="25" t="n"/>
+      <c r="E63" s="17" t="n"/>
+      <c r="F63" s="17" t="n"/>
+      <c r="G63" s="17" t="n"/>
+      <c r="H63" s="17" t="n"/>
+      <c r="I63" s="18" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
@@ -2245,11 +2317,11 @@
           <t>Kiểu kết quả chưa có truy vấn độc lập, xem lý do trong sheet Đối chiếu độc lập</t>
         </is>
       </c>
-      <c r="E64" s="25" t="n"/>
-      <c r="F64" s="25" t="n"/>
-      <c r="G64" s="25" t="n"/>
-      <c r="H64" s="25" t="n"/>
-      <c r="I64" s="25" t="n"/>
+      <c r="E64" s="17" t="n"/>
+      <c r="F64" s="17" t="n"/>
+      <c r="G64" s="17" t="n"/>
+      <c r="H64" s="17" t="n"/>
+      <c r="I64" s="18" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="24" t="inlineStr">
@@ -2287,9 +2359,9 @@
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A42:I42"/>
+    <mergeCell ref="D62:I62"/>
+    <mergeCell ref="A32:I32"/>
     <mergeCell ref="B50:I50"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="D62:I62"/>
     <mergeCell ref="E28:I28"/>
     <mergeCell ref="A22:I22"/>
     <mergeCell ref="A35:I35"/>
@@ -5508,17 +5580,17 @@
           <t>Backtest là gì</t>
         </is>
       </c>
-      <c r="N18" s="23" t="n"/>
+      <c r="N18" s="18" t="n"/>
       <c r="O18" s="22" t="inlineStr">
         <is>
           <t>Lùi về quá khứ giả vờ chưa biết tương lai, dự báo, rồi so với số thật đã ghi nhận. Cho biết dự báo sai bao nhiêu nếu dùng thật.</t>
         </is>
       </c>
-      <c r="P18" s="23" t="n"/>
-      <c r="Q18" s="23" t="n"/>
-      <c r="R18" s="23" t="n"/>
-      <c r="S18" s="23" t="n"/>
-      <c r="T18" s="23" t="n"/>
+      <c r="P18" s="17" t="n"/>
+      <c r="Q18" s="17" t="n"/>
+      <c r="R18" s="17" t="n"/>
+      <c r="S18" s="17" t="n"/>
+      <c r="T18" s="18" t="n"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -5564,17 +5636,17 @@
           <t>Gốc dự báo</t>
         </is>
       </c>
-      <c r="N19" s="23" t="n"/>
+      <c r="N19" s="18" t="n"/>
       <c r="O19" s="22" t="inlineStr">
         <is>
           <t>Tháng cuối cùng của phần lịch sử được dùng để dự báo (mỗi gốc cần ít nhất 24 tháng lịch sử).</t>
         </is>
       </c>
-      <c r="P19" s="23" t="n"/>
-      <c r="Q19" s="23" t="n"/>
-      <c r="R19" s="23" t="n"/>
-      <c r="S19" s="23" t="n"/>
-      <c r="T19" s="23" t="n"/>
+      <c r="P19" s="17" t="n"/>
+      <c r="Q19" s="17" t="n"/>
+      <c r="R19" s="17" t="n"/>
+      <c r="S19" s="17" t="n"/>
+      <c r="T19" s="18" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -5620,17 +5692,17 @@
           <t>Chân trời</t>
         </is>
       </c>
-      <c r="N20" s="23" t="n"/>
+      <c r="N20" s="18" t="n"/>
       <c r="O20" s="22" t="inlineStr">
         <is>
           <t>Dự báo cho tháng thứ mấy sau gốc: 1 là tháng kế tiếp, 6 là tháng thứ sáu.</t>
         </is>
       </c>
-      <c r="P20" s="23" t="n"/>
-      <c r="Q20" s="23" t="n"/>
-      <c r="R20" s="23" t="n"/>
-      <c r="S20" s="23" t="n"/>
-      <c r="T20" s="23" t="n"/>
+      <c r="P20" s="17" t="n"/>
+      <c r="Q20" s="17" t="n"/>
+      <c r="R20" s="17" t="n"/>
+      <c r="S20" s="17" t="n"/>
+      <c r="T20" s="18" t="n"/>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -5676,17 +5748,17 @@
           <t>ETS</t>
         </is>
       </c>
-      <c r="N21" s="23" t="n"/>
+      <c r="N21" s="18" t="n"/>
       <c r="O21" s="22" t="inlineStr">
         <is>
           <t>Phương pháp dự báo của hệ thống (làm trơn hàm mũ), kèm cận dưới và cận trên của khoảng tin cậy 95%.</t>
         </is>
       </c>
-      <c r="P21" s="23" t="n"/>
-      <c r="Q21" s="23" t="n"/>
-      <c r="R21" s="23" t="n"/>
-      <c r="S21" s="23" t="n"/>
-      <c r="T21" s="23" t="n"/>
+      <c r="P21" s="17" t="n"/>
+      <c r="Q21" s="17" t="n"/>
+      <c r="R21" s="17" t="n"/>
+      <c r="S21" s="17" t="n"/>
+      <c r="T21" s="18" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -5732,17 +5804,17 @@
           <t>Naive</t>
         </is>
       </c>
-      <c r="N22" s="23" t="n"/>
+      <c r="N22" s="18" t="n"/>
       <c r="O22" s="22" t="inlineStr">
         <is>
           <t>Phương pháp đơn giản: dự báo bằng đúng giá trị của tháng gần nhất.</t>
         </is>
       </c>
-      <c r="P22" s="23" t="n"/>
-      <c r="Q22" s="23" t="n"/>
-      <c r="R22" s="23" t="n"/>
-      <c r="S22" s="23" t="n"/>
-      <c r="T22" s="23" t="n"/>
+      <c r="P22" s="17" t="n"/>
+      <c r="Q22" s="17" t="n"/>
+      <c r="R22" s="17" t="n"/>
+      <c r="S22" s="17" t="n"/>
+      <c r="T22" s="18" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -5788,17 +5860,17 @@
           <t>Seasonal naive</t>
         </is>
       </c>
-      <c r="N23" s="23" t="n"/>
+      <c r="N23" s="18" t="n"/>
       <c r="O23" s="22" t="inlineStr">
         <is>
           <t>Dự báo bằng giá trị của cùng tháng năm trước.</t>
         </is>
       </c>
-      <c r="P23" s="23" t="n"/>
-      <c r="Q23" s="23" t="n"/>
-      <c r="R23" s="23" t="n"/>
-      <c r="S23" s="23" t="n"/>
-      <c r="T23" s="23" t="n"/>
+      <c r="P23" s="17" t="n"/>
+      <c r="Q23" s="17" t="n"/>
+      <c r="R23" s="17" t="n"/>
+      <c r="S23" s="17" t="n"/>
+      <c r="T23" s="18" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -5844,17 +5916,17 @@
           <t>Trung bình 3 tháng</t>
         </is>
       </c>
-      <c r="N24" s="23" t="n"/>
+      <c r="N24" s="18" t="n"/>
       <c r="O24" s="22" t="inlineStr">
         <is>
           <t>Dự báo bằng trung bình của 3 tháng gần nhất.</t>
         </is>
       </c>
-      <c r="P24" s="23" t="n"/>
-      <c r="Q24" s="23" t="n"/>
-      <c r="R24" s="23" t="n"/>
-      <c r="S24" s="23" t="n"/>
-      <c r="T24" s="23" t="n"/>
+      <c r="P24" s="17" t="n"/>
+      <c r="Q24" s="17" t="n"/>
+      <c r="R24" s="17" t="n"/>
+      <c r="S24" s="17" t="n"/>
+      <c r="T24" s="18" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
@@ -5900,17 +5972,17 @@
           <t>WAPE</t>
         </is>
       </c>
-      <c r="N25" s="23" t="n"/>
+      <c r="N25" s="18" t="n"/>
       <c r="O25" s="22" t="inlineStr">
         <is>
           <t>Sai số theo phần trăm: tổng độ lệch tuyệt đối chia tổng giá trị thật. 20% nghĩa là dự báo lệch trung bình khoảng 20% so với số thật; càng thấp càng tốt. Dùng để so ETS với các phương pháp đơn giản.</t>
         </is>
       </c>
-      <c r="P25" s="23" t="n"/>
-      <c r="Q25" s="23" t="n"/>
-      <c r="R25" s="23" t="n"/>
-      <c r="S25" s="23" t="n"/>
-      <c r="T25" s="23" t="n"/>
+      <c r="P25" s="17" t="n"/>
+      <c r="Q25" s="17" t="n"/>
+      <c r="R25" s="17" t="n"/>
+      <c r="S25" s="17" t="n"/>
+      <c r="T25" s="18" t="n"/>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -5956,17 +6028,17 @@
           <t>Phủ khoảng 95%</t>
         </is>
       </c>
-      <c r="N26" s="23" t="n"/>
+      <c r="N26" s="18" t="n"/>
       <c r="O26" s="22" t="inlineStr">
         <is>
           <t>Tỷ lệ số thật nằm trong khoảng tin cậy 95% mà hệ thống đưa ra. Nếu khoảng chuẩn thì khoảng 95%; thấp hơn nghĩa là khoảng đưa ra hẹp hơn thực tế.</t>
         </is>
       </c>
-      <c r="P26" s="23" t="n"/>
-      <c r="Q26" s="23" t="n"/>
-      <c r="R26" s="23" t="n"/>
-      <c r="S26" s="23" t="n"/>
-      <c r="T26" s="23" t="n"/>
+      <c r="P26" s="17" t="n"/>
+      <c r="Q26" s="17" t="n"/>
+      <c r="R26" s="17" t="n"/>
+      <c r="S26" s="17" t="n"/>
+      <c r="T26" s="18" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
@@ -6012,17 +6084,17 @@
           <t>Số mẫu</t>
         </is>
       </c>
-      <c r="N27" s="23" t="n"/>
+      <c r="N27" s="18" t="n"/>
       <c r="O27" s="22" t="inlineStr">
         <is>
           <t>Số cặp (gốc, chân trời) dùng để tính. Số mẫu nhỏ thì kết luận kém chắc chắn.</t>
         </is>
       </c>
-      <c r="P27" s="23" t="n"/>
-      <c r="Q27" s="23" t="n"/>
-      <c r="R27" s="23" t="n"/>
-      <c r="S27" s="23" t="n"/>
-      <c r="T27" s="23" t="n"/>
+      <c r="P27" s="17" t="n"/>
+      <c r="Q27" s="17" t="n"/>
+      <c r="R27" s="17" t="n"/>
+      <c r="S27" s="17" t="n"/>
+      <c r="T27" s="18" t="n"/>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -6068,17 +6140,17 @@
           <t>Cách kết luận</t>
         </is>
       </c>
-      <c r="N28" s="23" t="n"/>
+      <c r="N28" s="18" t="n"/>
       <c r="O28" s="22" t="inlineStr">
         <is>
           <t>Nếu WAPE của ETS xấp xỉ các phương pháp đơn giản thì ETS không hơn gì cách đơn giản. Dữ liệu này mô phỏng và ngắn nên chỉ để tham khảo.</t>
         </is>
       </c>
-      <c r="P28" s="23" t="n"/>
-      <c r="Q28" s="23" t="n"/>
-      <c r="R28" s="23" t="n"/>
-      <c r="S28" s="23" t="n"/>
-      <c r="T28" s="23" t="n"/>
+      <c r="P28" s="17" t="n"/>
+      <c r="Q28" s="17" t="n"/>
+      <c r="R28" s="17" t="n"/>
+      <c r="S28" s="17" t="n"/>
+      <c r="T28" s="18" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -10058,10 +10130,10 @@
           <t>Một loại yêu cầu mà backend gửi cho dịch vụ AI bên ngoài.</t>
         </is>
       </c>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="23" t="n"/>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="23" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18" t="n"/>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
@@ -10074,10 +10146,10 @@
           <t>Dữ liệu rời khỏi hệ thống trong lời gọi đó, và dữ liệu không bao giờ gửi (ví dụ dòng kết quả, mật khẩu, khóa).</t>
         </is>
       </c>
-      <c r="C21" s="23" t="n"/>
-      <c r="D21" s="23" t="n"/>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="23" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="18" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="21" t="inlineStr">
@@ -10090,10 +10162,10 @@
           <t>Biến cấu hình bật hoặc tắt việc gửi; mặc định thường là tắt.</t>
         </is>
       </c>
-      <c r="C22" s="23" t="n"/>
-      <c r="D22" s="23" t="n"/>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="23" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="18" t="n"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
@@ -10106,10 +10178,10 @@
           <t>Lời gọi này đang dùng hay không trên bản demo hiện tại.</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="23" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="23" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -11271,10 +11343,10 @@
           <t>Các hệ số tự đặt (ô chữ xanh): tỷ giá, hệ số token, hệ số suy nghĩ, tỷ lệ cache. Đổi ô thì cả bảng tự tính lại.</t>
         </is>
       </c>
-      <c r="C76" s="23" t="n"/>
-      <c r="D76" s="23" t="n"/>
-      <c r="E76" s="23" t="n"/>
-      <c r="F76" s="23" t="n"/>
+      <c r="C76" s="17" t="n"/>
+      <c r="D76" s="17" t="n"/>
+      <c r="E76" s="17" t="n"/>
+      <c r="F76" s="18" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="21" t="inlineStr">
@@ -11287,10 +11359,10 @@
           <t>Giá mỗi một triệu token (đơn vị tính tiền của dịch vụ AI) cho phần đọc vào (đầu vào) và phần AI viết ra (đầu ra).</t>
         </is>
       </c>
-      <c r="C77" s="23" t="n"/>
-      <c r="D77" s="23" t="n"/>
-      <c r="E77" s="23" t="n"/>
-      <c r="F77" s="23" t="n"/>
+      <c r="C77" s="17" t="n"/>
+      <c r="D77" s="17" t="n"/>
+      <c r="E77" s="17" t="n"/>
+      <c r="F77" s="18" t="n"/>
     </row>
     <row r="78" ht="32" customHeight="1">
       <c r="A78" s="21" t="inlineStr">
@@ -11303,10 +11375,10 @@
           <t>Số token đo trên lời nhắc thật của hệ thống. Số lời gọi mỗi câu là mỗi câu hỏi trung bình gọi AI bao nhiêu lần: cột đo trên bộ test (0,47 lần vì nhiều câu không cần AI) và cột kịch bản xấu (mọi câu đều gọi AI).</t>
         </is>
       </c>
-      <c r="C78" s="23" t="n"/>
-      <c r="D78" s="23" t="n"/>
-      <c r="E78" s="23" t="n"/>
-      <c r="F78" s="23" t="n"/>
+      <c r="C78" s="17" t="n"/>
+      <c r="D78" s="17" t="n"/>
+      <c r="E78" s="17" t="n"/>
+      <c r="F78" s="18" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="21" t="inlineStr">
@@ -11319,10 +11391,10 @@
           <t>Tiền phải trả cho 1.000 câu hỏi theo từng mô hình. Có cache là khi phần lời nhắc lặp lại được tính giá rẻ hơn.</t>
         </is>
       </c>
-      <c r="C79" s="23" t="n"/>
-      <c r="D79" s="23" t="n"/>
-      <c r="E79" s="23" t="n"/>
-      <c r="F79" s="23" t="n"/>
+      <c r="C79" s="17" t="n"/>
+      <c r="D79" s="17" t="n"/>
+      <c r="E79" s="17" t="n"/>
+      <c r="F79" s="18" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="21" t="inlineStr">
@@ -11335,10 +11407,10 @@
           <t>Chi phí D nhân với số câu hỏi mỗi tháng (ô số câu nhập tay được).</t>
         </is>
       </c>
-      <c r="C80" s="23" t="n"/>
-      <c r="D80" s="23" t="n"/>
-      <c r="E80" s="23" t="n"/>
-      <c r="F80" s="23" t="n"/>
+      <c r="C80" s="17" t="n"/>
+      <c r="D80" s="17" t="n"/>
+      <c r="E80" s="17" t="n"/>
+      <c r="F80" s="18" t="n"/>
     </row>
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="21" t="inlineStr">
@@ -11351,10 +11423,10 @@
           <t>Giá thuê máy chủ có card đồ họa để chạy mô hình offline; cố định theo tháng, không phụ thuộc số câu hỏi. Chưa gồm nhân sự.</t>
         </is>
       </c>
-      <c r="C81" s="23" t="n"/>
-      <c r="D81" s="23" t="n"/>
-      <c r="E81" s="23" t="n"/>
-      <c r="F81" s="23" t="n"/>
+      <c r="C81" s="17" t="n"/>
+      <c r="D81" s="17" t="n"/>
+      <c r="E81" s="17" t="n"/>
+      <c r="F81" s="18" t="n"/>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="21" t="inlineStr">
@@ -11367,10 +11439,10 @@
           <t>Số câu hỏi mỗi tháng mà tại đó dùng API và thuê máy chủ tốn như nhau. Ít hơn mức này thì API rẻ hơn.</t>
         </is>
       </c>
-      <c r="C82" s="23" t="n"/>
-      <c r="D82" s="23" t="n"/>
-      <c r="E82" s="23" t="n"/>
-      <c r="F82" s="23" t="n"/>
+      <c r="C82" s="17" t="n"/>
+      <c r="D82" s="17" t="n"/>
+      <c r="E82" s="17" t="n"/>
+      <c r="F82" s="18" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="21" t="inlineStr">
@@ -11383,10 +11455,10 @@
           <t>Những điều tiền không nói hết: chất lượng, độ trễ, riêng tư, vận hành.</t>
         </is>
       </c>
-      <c r="C83" s="23" t="n"/>
-      <c r="D83" s="23" t="n"/>
-      <c r="E83" s="23" t="n"/>
-      <c r="F83" s="23" t="n"/>
+      <c r="C83" s="17" t="n"/>
+      <c r="D83" s="17" t="n"/>
+      <c r="E83" s="17" t="n"/>
+      <c r="F83" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -13396,18 +13468,18 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B29" s="23" t="n"/>
-      <c r="C29" s="23" t="n"/>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="18" t="n"/>
       <c r="D29" s="22" t="inlineStr">
         <is>
           <t>Mã của ca kiểm thử (ví dụ R01, H12, M3). Dùng mã này để tìm lại ca trong kịch bản chạy và trong báo cáo.</t>
         </is>
       </c>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="23" t="n"/>
-      <c r="H29" s="23" t="n"/>
-      <c r="I29" s="23" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="17" t="n"/>
+      <c r="H29" s="17" t="n"/>
+      <c r="I29" s="18" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="21" t="inlineStr">
@@ -13415,18 +13487,18 @@
           <t>Test Suite</t>
         </is>
       </c>
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="18" t="n"/>
       <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Nhóm (bộ) kiểm thử mà ca thuộc về.</t>
         </is>
       </c>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="23" t="n"/>
-      <c r="I30" s="23" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
+      <c r="H30" s="17" t="n"/>
+      <c r="I30" s="18" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="21" t="inlineStr">
@@ -13434,18 +13506,18 @@
           <t>Tiêu đề (Title)</t>
         </is>
       </c>
-      <c r="B31" s="23" t="n"/>
-      <c r="C31" s="23" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="18" t="n"/>
       <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Tên ngắn của ca: câu hỏi chính được đem ra thử.</t>
         </is>
       </c>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="23" t="n"/>
-      <c r="H31" s="23" t="n"/>
-      <c r="I31" s="23" t="n"/>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="17" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="18" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="21" t="inlineStr">
@@ -13453,18 +13525,18 @@
           <t>Điều kiện tiên quyết (Pre-conditions)</t>
         </is>
       </c>
-      <c r="B32" s="23" t="n"/>
-      <c r="C32" s="23" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="18" t="n"/>
       <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Cần có gì trước khi chạy: đăng nhập bằng vai trò nào, ngôn ngữ nào, hội thoại mới hay nhiều lượt trong cùng một hội thoại.</t>
         </is>
       </c>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="23" t="n"/>
-      <c r="H32" s="23" t="n"/>
-      <c r="I32" s="23" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="18" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="21" t="inlineStr">
@@ -13472,18 +13544,18 @@
           <t>Các bước (Test Steps)</t>
         </is>
       </c>
-      <c r="B33" s="23" t="n"/>
-      <c r="C33" s="23" t="n"/>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="18" t="n"/>
       <c r="D33" s="22" t="inlineStr">
         <is>
           <t>Việc đã làm, theo thứ tự: gửi từng câu hỏi, rồi (nếu có) chạy một câu SQL độc lập trên kho dữ liệu để đối chiếu số.</t>
         </is>
       </c>
-      <c r="E33" s="23" t="n"/>
-      <c r="F33" s="23" t="n"/>
-      <c r="G33" s="23" t="n"/>
-      <c r="H33" s="23" t="n"/>
-      <c r="I33" s="23" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="18" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="21" t="inlineStr">
@@ -13491,18 +13563,18 @@
           <t>Dữ liệu kiểm thử (Test Data)</t>
         </is>
       </c>
-      <c r="B34" s="23" t="n"/>
-      <c r="C34" s="23" t="n"/>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="18" t="n"/>
       <c r="D34" s="22" t="inlineStr">
         <is>
           <t>Nguyên văn các câu hỏi đã gửi cho hệ thống.</t>
         </is>
       </c>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="23" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="17" t="n"/>
+      <c r="H34" s="17" t="n"/>
+      <c r="I34" s="18" t="n"/>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="21" t="inlineStr">
@@ -13510,18 +13582,18 @@
           <t>Kết quả mong đợi (Expected Result)</t>
         </is>
       </c>
-      <c r="B35" s="23" t="n"/>
-      <c r="C35" s="23" t="n"/>
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="18" t="n"/>
       <c r="D35" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống phải làm để ca được coi là đạt: trạng thái cho phép (ok = có số liệu, needs_clarification = hỏi lại, denied = từ chối, no_data = không có dữ liệu), số dòng, loại biểu đồ, cụm chữ phải có hoặc không được có, và số có khớp kho dữ liệu hay không.</t>
         </is>
       </c>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="23" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="17" t="n"/>
+      <c r="H35" s="17" t="n"/>
+      <c r="I35" s="18" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="21" t="inlineStr">
@@ -13529,18 +13601,18 @@
           <t>Kết quả thực tế (Actual Result)</t>
         </is>
       </c>
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="18" t="n"/>
       <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống đã trả về: trạng thái, câu trả lời nguyên văn (cắt ngắn), số dòng của bảng và loại biểu đồ.</t>
         </is>
       </c>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="23" t="n"/>
-      <c r="I36" s="23" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17" t="n"/>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="18" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="21" t="inlineStr">
@@ -13548,18 +13620,18 @@
           <t>Trạng thái (Status)</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n"/>
-      <c r="C37" s="23" t="n"/>
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="18" t="n"/>
       <c r="D37" s="22" t="inlineStr">
         <is>
           <t>Passed = đạt mọi yêu cầu. Failed = có yêu cầu sai. Blocked = không chạy được vì dịch vụ AI báo bận (hết hạn mức), không phải lỗi của hệ thống. Not Run = chưa chạy.</t>
         </is>
       </c>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="23" t="n"/>
-      <c r="I37" s="23" t="n"/>
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="17" t="n"/>
+      <c r="H37" s="17" t="n"/>
+      <c r="I37" s="18" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="21" t="inlineStr">
@@ -13567,18 +13639,18 @@
           <t>Lần chạy đầu (First run)</t>
         </is>
       </c>
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="18" t="n"/>
       <c r="D38" s="22" t="inlineStr">
         <is>
           <t>Kết quả ở lần chạy đầu tiên. Ca báo Blocked ở lần đầu được chạy lại cho đến khi không còn báo bận, nên cột Trạng thái là kết quả cuối còn cột này giữ dấu vết lần đầu.</t>
         </is>
       </c>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="23" t="n"/>
-      <c r="I38" s="23" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="17" t="n"/>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="18" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="21" t="inlineStr">
@@ -13586,18 +13658,18 @@
           <t>Người thực hiện / Ngày</t>
         </is>
       </c>
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="18" t="n"/>
       <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Ai hoặc cái gì chạy ca (kịch bản tự động) và chạy ngày nào.</t>
         </is>
       </c>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="23" t="n"/>
-      <c r="H39" s="23" t="n"/>
-      <c r="I39" s="23" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="18" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="21" t="inlineStr">
@@ -13605,18 +13677,18 @@
           <t>Ghi chú và bằng chứng (Comments)</t>
         </is>
       </c>
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="18" t="n"/>
       <c r="D40" s="22" t="inlineStr">
         <is>
           <t>Bằng chứng cho kết quả: câu SQL độc lập chạy trên kho dữ liệu, tham số và kết quả của nó (để so với con số trong câu trả lời). Với tin nhắn nhiều yêu cầu: kết quả từng phần.</t>
         </is>
       </c>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="18" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="21" t="inlineStr">
@@ -13624,18 +13696,18 @@
           <t>Ảnh trình duyệt (Screenshot)</t>
         </is>
       </c>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
+      <c r="B41" s="17" t="n"/>
+      <c r="C41" s="18" t="n"/>
       <c r="D41" s="22" t="inlineStr">
         <is>
           <t>Ảnh chụp trang web thật sau khi hỏi đúng câu này (chỉ sheet RAG).</t>
         </is>
       </c>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
-      <c r="I41" s="23" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="17" t="n"/>
+      <c r="G41" s="17" t="n"/>
+      <c r="H41" s="17" t="n"/>
+      <c r="I41" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -20068,18 +20140,18 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B95" s="23" t="n"/>
-      <c r="C95" s="23" t="n"/>
+      <c r="B95" s="17" t="n"/>
+      <c r="C95" s="18" t="n"/>
       <c r="D95" s="22" t="inlineStr">
         <is>
           <t>Mã của ca kiểm thử (ví dụ R01, H12, M3). Dùng mã này để tìm lại ca trong kịch bản chạy và trong báo cáo.</t>
         </is>
       </c>
-      <c r="E95" s="23" t="n"/>
-      <c r="F95" s="23" t="n"/>
-      <c r="G95" s="23" t="n"/>
-      <c r="H95" s="23" t="n"/>
-      <c r="I95" s="23" t="n"/>
+      <c r="E95" s="17" t="n"/>
+      <c r="F95" s="17" t="n"/>
+      <c r="G95" s="17" t="n"/>
+      <c r="H95" s="17" t="n"/>
+      <c r="I95" s="18" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="21" t="inlineStr">
@@ -20087,18 +20159,18 @@
           <t>Test Suite</t>
         </is>
       </c>
-      <c r="B96" s="23" t="n"/>
-      <c r="C96" s="23" t="n"/>
+      <c r="B96" s="17" t="n"/>
+      <c r="C96" s="18" t="n"/>
       <c r="D96" s="22" t="inlineStr">
         <is>
           <t>Nhóm (bộ) kiểm thử mà ca thuộc về.</t>
         </is>
       </c>
-      <c r="E96" s="23" t="n"/>
-      <c r="F96" s="23" t="n"/>
-      <c r="G96" s="23" t="n"/>
-      <c r="H96" s="23" t="n"/>
-      <c r="I96" s="23" t="n"/>
+      <c r="E96" s="17" t="n"/>
+      <c r="F96" s="17" t="n"/>
+      <c r="G96" s="17" t="n"/>
+      <c r="H96" s="17" t="n"/>
+      <c r="I96" s="18" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="21" t="inlineStr">
@@ -20106,18 +20178,18 @@
           <t>Tiêu đề (Title)</t>
         </is>
       </c>
-      <c r="B97" s="23" t="n"/>
-      <c r="C97" s="23" t="n"/>
+      <c r="B97" s="17" t="n"/>
+      <c r="C97" s="18" t="n"/>
       <c r="D97" s="22" t="inlineStr">
         <is>
           <t>Tên ngắn của ca: câu hỏi chính được đem ra thử.</t>
         </is>
       </c>
-      <c r="E97" s="23" t="n"/>
-      <c r="F97" s="23" t="n"/>
-      <c r="G97" s="23" t="n"/>
-      <c r="H97" s="23" t="n"/>
-      <c r="I97" s="23" t="n"/>
+      <c r="E97" s="17" t="n"/>
+      <c r="F97" s="17" t="n"/>
+      <c r="G97" s="17" t="n"/>
+      <c r="H97" s="17" t="n"/>
+      <c r="I97" s="18" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="21" t="inlineStr">
@@ -20125,18 +20197,18 @@
           <t>Điều kiện tiên quyết (Pre-conditions)</t>
         </is>
       </c>
-      <c r="B98" s="23" t="n"/>
-      <c r="C98" s="23" t="n"/>
+      <c r="B98" s="17" t="n"/>
+      <c r="C98" s="18" t="n"/>
       <c r="D98" s="22" t="inlineStr">
         <is>
           <t>Cần có gì trước khi chạy: đăng nhập bằng vai trò nào, ngôn ngữ nào, hội thoại mới hay nhiều lượt trong cùng một hội thoại.</t>
         </is>
       </c>
-      <c r="E98" s="23" t="n"/>
-      <c r="F98" s="23" t="n"/>
-      <c r="G98" s="23" t="n"/>
-      <c r="H98" s="23" t="n"/>
-      <c r="I98" s="23" t="n"/>
+      <c r="E98" s="17" t="n"/>
+      <c r="F98" s="17" t="n"/>
+      <c r="G98" s="17" t="n"/>
+      <c r="H98" s="17" t="n"/>
+      <c r="I98" s="18" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="21" t="inlineStr">
@@ -20144,18 +20216,18 @@
           <t>Các bước (Test Steps)</t>
         </is>
       </c>
-      <c r="B99" s="23" t="n"/>
-      <c r="C99" s="23" t="n"/>
+      <c r="B99" s="17" t="n"/>
+      <c r="C99" s="18" t="n"/>
       <c r="D99" s="22" t="inlineStr">
         <is>
           <t>Việc đã làm, theo thứ tự: gửi từng câu hỏi, rồi (nếu có) chạy một câu SQL độc lập trên kho dữ liệu để đối chiếu số.</t>
         </is>
       </c>
-      <c r="E99" s="23" t="n"/>
-      <c r="F99" s="23" t="n"/>
-      <c r="G99" s="23" t="n"/>
-      <c r="H99" s="23" t="n"/>
-      <c r="I99" s="23" t="n"/>
+      <c r="E99" s="17" t="n"/>
+      <c r="F99" s="17" t="n"/>
+      <c r="G99" s="17" t="n"/>
+      <c r="H99" s="17" t="n"/>
+      <c r="I99" s="18" t="n"/>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="21" t="inlineStr">
@@ -20163,18 +20235,18 @@
           <t>Dữ liệu kiểm thử (Test Data)</t>
         </is>
       </c>
-      <c r="B100" s="23" t="n"/>
-      <c r="C100" s="23" t="n"/>
+      <c r="B100" s="17" t="n"/>
+      <c r="C100" s="18" t="n"/>
       <c r="D100" s="22" t="inlineStr">
         <is>
           <t>Nguyên văn các câu hỏi đã gửi cho hệ thống.</t>
         </is>
       </c>
-      <c r="E100" s="23" t="n"/>
-      <c r="F100" s="23" t="n"/>
-      <c r="G100" s="23" t="n"/>
-      <c r="H100" s="23" t="n"/>
-      <c r="I100" s="23" t="n"/>
+      <c r="E100" s="17" t="n"/>
+      <c r="F100" s="17" t="n"/>
+      <c r="G100" s="17" t="n"/>
+      <c r="H100" s="17" t="n"/>
+      <c r="I100" s="18" t="n"/>
     </row>
     <row r="101" ht="32" customHeight="1">
       <c r="A101" s="21" t="inlineStr">
@@ -20182,18 +20254,18 @@
           <t>Kết quả mong đợi (Expected Result)</t>
         </is>
       </c>
-      <c r="B101" s="23" t="n"/>
-      <c r="C101" s="23" t="n"/>
+      <c r="B101" s="17" t="n"/>
+      <c r="C101" s="18" t="n"/>
       <c r="D101" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống phải làm để ca được coi là đạt: trạng thái cho phép (ok = có số liệu, needs_clarification = hỏi lại, denied = từ chối, no_data = không có dữ liệu), số dòng, loại biểu đồ, cụm chữ phải có hoặc không được có, và số có khớp kho dữ liệu hay không.</t>
         </is>
       </c>
-      <c r="E101" s="23" t="n"/>
-      <c r="F101" s="23" t="n"/>
-      <c r="G101" s="23" t="n"/>
-      <c r="H101" s="23" t="n"/>
-      <c r="I101" s="23" t="n"/>
+      <c r="E101" s="17" t="n"/>
+      <c r="F101" s="17" t="n"/>
+      <c r="G101" s="17" t="n"/>
+      <c r="H101" s="17" t="n"/>
+      <c r="I101" s="18" t="n"/>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="21" t="inlineStr">
@@ -20201,18 +20273,18 @@
           <t>Kết quả thực tế (Actual Result)</t>
         </is>
       </c>
-      <c r="B102" s="23" t="n"/>
-      <c r="C102" s="23" t="n"/>
+      <c r="B102" s="17" t="n"/>
+      <c r="C102" s="18" t="n"/>
       <c r="D102" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống đã trả về: trạng thái, câu trả lời nguyên văn (cắt ngắn), số dòng của bảng và loại biểu đồ.</t>
         </is>
       </c>
-      <c r="E102" s="23" t="n"/>
-      <c r="F102" s="23" t="n"/>
-      <c r="G102" s="23" t="n"/>
-      <c r="H102" s="23" t="n"/>
-      <c r="I102" s="23" t="n"/>
+      <c r="E102" s="17" t="n"/>
+      <c r="F102" s="17" t="n"/>
+      <c r="G102" s="17" t="n"/>
+      <c r="H102" s="17" t="n"/>
+      <c r="I102" s="18" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="21" t="inlineStr">
@@ -20220,18 +20292,18 @@
           <t>Trạng thái (Status)</t>
         </is>
       </c>
-      <c r="B103" s="23" t="n"/>
-      <c r="C103" s="23" t="n"/>
+      <c r="B103" s="17" t="n"/>
+      <c r="C103" s="18" t="n"/>
       <c r="D103" s="22" t="inlineStr">
         <is>
           <t>Passed = đạt mọi yêu cầu. Failed = có yêu cầu sai. Blocked = không chạy được vì dịch vụ AI báo bận (hết hạn mức), không phải lỗi của hệ thống. Not Run = chưa chạy.</t>
         </is>
       </c>
-      <c r="E103" s="23" t="n"/>
-      <c r="F103" s="23" t="n"/>
-      <c r="G103" s="23" t="n"/>
-      <c r="H103" s="23" t="n"/>
-      <c r="I103" s="23" t="n"/>
+      <c r="E103" s="17" t="n"/>
+      <c r="F103" s="17" t="n"/>
+      <c r="G103" s="17" t="n"/>
+      <c r="H103" s="17" t="n"/>
+      <c r="I103" s="18" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="21" t="inlineStr">
@@ -20239,18 +20311,18 @@
           <t>Lần chạy đầu (First run)</t>
         </is>
       </c>
-      <c r="B104" s="23" t="n"/>
-      <c r="C104" s="23" t="n"/>
+      <c r="B104" s="17" t="n"/>
+      <c r="C104" s="18" t="n"/>
       <c r="D104" s="22" t="inlineStr">
         <is>
           <t>Kết quả ở lần chạy đầu tiên. Ca báo Blocked ở lần đầu được chạy lại cho đến khi không còn báo bận, nên cột Trạng thái là kết quả cuối còn cột này giữ dấu vết lần đầu.</t>
         </is>
       </c>
-      <c r="E104" s="23" t="n"/>
-      <c r="F104" s="23" t="n"/>
-      <c r="G104" s="23" t="n"/>
-      <c r="H104" s="23" t="n"/>
-      <c r="I104" s="23" t="n"/>
+      <c r="E104" s="17" t="n"/>
+      <c r="F104" s="17" t="n"/>
+      <c r="G104" s="17" t="n"/>
+      <c r="H104" s="17" t="n"/>
+      <c r="I104" s="18" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="21" t="inlineStr">
@@ -20258,18 +20330,18 @@
           <t>Người thực hiện / Ngày</t>
         </is>
       </c>
-      <c r="B105" s="23" t="n"/>
-      <c r="C105" s="23" t="n"/>
+      <c r="B105" s="17" t="n"/>
+      <c r="C105" s="18" t="n"/>
       <c r="D105" s="22" t="inlineStr">
         <is>
           <t>Ai hoặc cái gì chạy ca (kịch bản tự động) và chạy ngày nào.</t>
         </is>
       </c>
-      <c r="E105" s="23" t="n"/>
-      <c r="F105" s="23" t="n"/>
-      <c r="G105" s="23" t="n"/>
-      <c r="H105" s="23" t="n"/>
-      <c r="I105" s="23" t="n"/>
+      <c r="E105" s="17" t="n"/>
+      <c r="F105" s="17" t="n"/>
+      <c r="G105" s="17" t="n"/>
+      <c r="H105" s="17" t="n"/>
+      <c r="I105" s="18" t="n"/>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="21" t="inlineStr">
@@ -20277,18 +20349,18 @@
           <t>Ghi chú và bằng chứng (Comments)</t>
         </is>
       </c>
-      <c r="B106" s="23" t="n"/>
-      <c r="C106" s="23" t="n"/>
+      <c r="B106" s="17" t="n"/>
+      <c r="C106" s="18" t="n"/>
       <c r="D106" s="22" t="inlineStr">
         <is>
           <t>Bằng chứng cho kết quả: câu SQL độc lập chạy trên kho dữ liệu, tham số và kết quả của nó (để so với con số trong câu trả lời). Với tin nhắn nhiều yêu cầu: kết quả từng phần.</t>
         </is>
       </c>
-      <c r="E106" s="23" t="n"/>
-      <c r="F106" s="23" t="n"/>
-      <c r="G106" s="23" t="n"/>
-      <c r="H106" s="23" t="n"/>
-      <c r="I106" s="23" t="n"/>
+      <c r="E106" s="17" t="n"/>
+      <c r="F106" s="17" t="n"/>
+      <c r="G106" s="17" t="n"/>
+      <c r="H106" s="17" t="n"/>
+      <c r="I106" s="18" t="n"/>
     </row>
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="21" t="inlineStr">
@@ -20296,18 +20368,18 @@
           <t>Nhiều lượt hỏi</t>
         </is>
       </c>
-      <c r="B107" s="23" t="n"/>
-      <c r="C107" s="23" t="n"/>
+      <c r="B107" s="17" t="n"/>
+      <c r="C107" s="18" t="n"/>
       <c r="D107" s="22" t="inlineStr">
         <is>
           <t>Ca có nhiều lượt: các lượt được đánh số trong cột Các bước, Dữ liệu, Mong đợi và Thực tế, theo cùng thứ tự.</t>
         </is>
       </c>
-      <c r="E107" s="23" t="n"/>
-      <c r="F107" s="23" t="n"/>
-      <c r="G107" s="23" t="n"/>
-      <c r="H107" s="23" t="n"/>
-      <c r="I107" s="23" t="n"/>
+      <c r="E107" s="17" t="n"/>
+      <c r="F107" s="17" t="n"/>
+      <c r="G107" s="17" t="n"/>
+      <c r="H107" s="17" t="n"/>
+      <c r="I107" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -23708,18 +23780,18 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
+      <c r="B52" s="17" t="n"/>
+      <c r="C52" s="18" t="n"/>
       <c r="D52" s="22" t="inlineStr">
         <is>
           <t>Mã của ca kiểm thử (ví dụ R01, H12, M3). Dùng mã này để tìm lại ca trong kịch bản chạy và trong báo cáo.</t>
         </is>
       </c>
-      <c r="E52" s="23" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="23" t="n"/>
-      <c r="I52" s="23" t="n"/>
+      <c r="E52" s="17" t="n"/>
+      <c r="F52" s="17" t="n"/>
+      <c r="G52" s="17" t="n"/>
+      <c r="H52" s="17" t="n"/>
+      <c r="I52" s="18" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="21" t="inlineStr">
@@ -23727,18 +23799,18 @@
           <t>Test Suite</t>
         </is>
       </c>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
+      <c r="B53" s="17" t="n"/>
+      <c r="C53" s="18" t="n"/>
       <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Nhóm (bộ) kiểm thử mà ca thuộc về.</t>
         </is>
       </c>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
+      <c r="E53" s="17" t="n"/>
+      <c r="F53" s="17" t="n"/>
+      <c r="G53" s="17" t="n"/>
+      <c r="H53" s="17" t="n"/>
+      <c r="I53" s="18" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="21" t="inlineStr">
@@ -23746,18 +23818,18 @@
           <t>Tiêu đề (Title)</t>
         </is>
       </c>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
+      <c r="B54" s="17" t="n"/>
+      <c r="C54" s="18" t="n"/>
       <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Tên ngắn của ca: câu hỏi chính được đem ra thử.</t>
         </is>
       </c>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="17" t="n"/>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="18" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="21" t="inlineStr">
@@ -23765,18 +23837,18 @@
           <t>Điều kiện tiên quyết (Pre-conditions)</t>
         </is>
       </c>
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
+      <c r="B55" s="17" t="n"/>
+      <c r="C55" s="18" t="n"/>
       <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Cần có gì trước khi chạy: đăng nhập bằng vai trò nào, ngôn ngữ nào, hội thoại mới hay nhiều lượt trong cùng một hội thoại.</t>
         </is>
       </c>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="23" t="n"/>
-      <c r="H55" s="23" t="n"/>
-      <c r="I55" s="23" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="17" t="n"/>
+      <c r="G55" s="17" t="n"/>
+      <c r="H55" s="17" t="n"/>
+      <c r="I55" s="18" t="n"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="21" t="inlineStr">
@@ -23784,18 +23856,18 @@
           <t>Các bước (Test Steps)</t>
         </is>
       </c>
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
+      <c r="B56" s="17" t="n"/>
+      <c r="C56" s="18" t="n"/>
       <c r="D56" s="22" t="inlineStr">
         <is>
           <t>Việc đã làm, theo thứ tự: gửi từng câu hỏi, rồi (nếu có) chạy một câu SQL độc lập trên kho dữ liệu để đối chiếu số.</t>
         </is>
       </c>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="23" t="n"/>
-      <c r="H56" s="23" t="n"/>
-      <c r="I56" s="23" t="n"/>
+      <c r="E56" s="17" t="n"/>
+      <c r="F56" s="17" t="n"/>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="18" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="21" t="inlineStr">
@@ -23803,18 +23875,18 @@
           <t>Dữ liệu kiểm thử (Test Data)</t>
         </is>
       </c>
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="18" t="n"/>
       <c r="D57" s="22" t="inlineStr">
         <is>
           <t>Nguyên văn các câu hỏi đã gửi cho hệ thống.</t>
         </is>
       </c>
-      <c r="E57" s="23" t="n"/>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="23" t="n"/>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="n"/>
+      <c r="E57" s="17" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="18" t="n"/>
     </row>
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="21" t="inlineStr">
@@ -23822,18 +23894,18 @@
           <t>Kết quả mong đợi (Expected Result)</t>
         </is>
       </c>
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
+      <c r="B58" s="17" t="n"/>
+      <c r="C58" s="18" t="n"/>
       <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống phải làm để ca được coi là đạt: trạng thái cho phép (ok = có số liệu, needs_clarification = hỏi lại, denied = từ chối, no_data = không có dữ liệu), số dòng, loại biểu đồ, cụm chữ phải có hoặc không được có, và số có khớp kho dữ liệu hay không.</t>
         </is>
       </c>
-      <c r="E58" s="23" t="n"/>
-      <c r="F58" s="23" t="n"/>
-      <c r="G58" s="23" t="n"/>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="23" t="n"/>
+      <c r="E58" s="17" t="n"/>
+      <c r="F58" s="17" t="n"/>
+      <c r="G58" s="17" t="n"/>
+      <c r="H58" s="17" t="n"/>
+      <c r="I58" s="18" t="n"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="21" t="inlineStr">
@@ -23841,18 +23913,18 @@
           <t>Kết quả thực tế (Actual Result)</t>
         </is>
       </c>
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
+      <c r="B59" s="17" t="n"/>
+      <c r="C59" s="18" t="n"/>
       <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống đã trả về: trạng thái, câu trả lời nguyên văn (cắt ngắn), số dòng của bảng và loại biểu đồ.</t>
         </is>
       </c>
-      <c r="E59" s="23" t="n"/>
-      <c r="F59" s="23" t="n"/>
-      <c r="G59" s="23" t="n"/>
-      <c r="H59" s="23" t="n"/>
-      <c r="I59" s="23" t="n"/>
+      <c r="E59" s="17" t="n"/>
+      <c r="F59" s="17" t="n"/>
+      <c r="G59" s="17" t="n"/>
+      <c r="H59" s="17" t="n"/>
+      <c r="I59" s="18" t="n"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="21" t="inlineStr">
@@ -23860,18 +23932,18 @@
           <t>Trạng thái (Status)</t>
         </is>
       </c>
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
+      <c r="B60" s="17" t="n"/>
+      <c r="C60" s="18" t="n"/>
       <c r="D60" s="22" t="inlineStr">
         <is>
           <t>Passed = đạt mọi yêu cầu. Failed = có yêu cầu sai. Blocked = không chạy được vì dịch vụ AI báo bận (hết hạn mức), không phải lỗi của hệ thống. Not Run = chưa chạy.</t>
         </is>
       </c>
-      <c r="E60" s="23" t="n"/>
-      <c r="F60" s="23" t="n"/>
-      <c r="G60" s="23" t="n"/>
-      <c r="H60" s="23" t="n"/>
-      <c r="I60" s="23" t="n"/>
+      <c r="E60" s="17" t="n"/>
+      <c r="F60" s="17" t="n"/>
+      <c r="G60" s="17" t="n"/>
+      <c r="H60" s="17" t="n"/>
+      <c r="I60" s="18" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="21" t="inlineStr">
@@ -23879,18 +23951,18 @@
           <t>Lần chạy đầu (First run)</t>
         </is>
       </c>
-      <c r="B61" s="23" t="n"/>
-      <c r="C61" s="23" t="n"/>
+      <c r="B61" s="17" t="n"/>
+      <c r="C61" s="18" t="n"/>
       <c r="D61" s="22" t="inlineStr">
         <is>
           <t>Kết quả ở lần chạy đầu tiên. Ca báo Blocked ở lần đầu được chạy lại cho đến khi không còn báo bận, nên cột Trạng thái là kết quả cuối còn cột này giữ dấu vết lần đầu.</t>
         </is>
       </c>
-      <c r="E61" s="23" t="n"/>
-      <c r="F61" s="23" t="n"/>
-      <c r="G61" s="23" t="n"/>
-      <c r="H61" s="23" t="n"/>
-      <c r="I61" s="23" t="n"/>
+      <c r="E61" s="17" t="n"/>
+      <c r="F61" s="17" t="n"/>
+      <c r="G61" s="17" t="n"/>
+      <c r="H61" s="17" t="n"/>
+      <c r="I61" s="18" t="n"/>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="21" t="inlineStr">
@@ -23898,18 +23970,18 @@
           <t>Người thực hiện / Ngày</t>
         </is>
       </c>
-      <c r="B62" s="23" t="n"/>
-      <c r="C62" s="23" t="n"/>
+      <c r="B62" s="17" t="n"/>
+      <c r="C62" s="18" t="n"/>
       <c r="D62" s="22" t="inlineStr">
         <is>
           <t>Ai hoặc cái gì chạy ca (kịch bản tự động) và chạy ngày nào.</t>
         </is>
       </c>
-      <c r="E62" s="23" t="n"/>
-      <c r="F62" s="23" t="n"/>
-      <c r="G62" s="23" t="n"/>
-      <c r="H62" s="23" t="n"/>
-      <c r="I62" s="23" t="n"/>
+      <c r="E62" s="17" t="n"/>
+      <c r="F62" s="17" t="n"/>
+      <c r="G62" s="17" t="n"/>
+      <c r="H62" s="17" t="n"/>
+      <c r="I62" s="18" t="n"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="21" t="inlineStr">
@@ -23917,18 +23989,18 @@
           <t>Ghi chú và bằng chứng (Comments)</t>
         </is>
       </c>
-      <c r="B63" s="23" t="n"/>
-      <c r="C63" s="23" t="n"/>
+      <c r="B63" s="17" t="n"/>
+      <c r="C63" s="18" t="n"/>
       <c r="D63" s="22" t="inlineStr">
         <is>
           <t>Bằng chứng cho kết quả: câu SQL độc lập chạy trên kho dữ liệu, tham số và kết quả của nó (để so với con số trong câu trả lời). Với tin nhắn nhiều yêu cầu: kết quả từng phần.</t>
         </is>
       </c>
-      <c r="E63" s="23" t="n"/>
-      <c r="F63" s="23" t="n"/>
-      <c r="G63" s="23" t="n"/>
-      <c r="H63" s="23" t="n"/>
-      <c r="I63" s="23" t="n"/>
+      <c r="E63" s="17" t="n"/>
+      <c r="F63" s="17" t="n"/>
+      <c r="G63" s="17" t="n"/>
+      <c r="H63" s="17" t="n"/>
+      <c r="I63" s="18" t="n"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="21" t="inlineStr">
@@ -23936,18 +24008,18 @@
           <t>Các phần của tin nhắn</t>
         </is>
       </c>
-      <c r="B64" s="23" t="n"/>
-      <c r="C64" s="23" t="n"/>
+      <c r="B64" s="17" t="n"/>
+      <c r="C64" s="18" t="n"/>
       <c r="D64" s="22" t="inlineStr">
         <is>
           <t>Một tin nhắn có nhiều yêu cầu được hệ thống tách thành các phần đánh số; kết quả từng phần nằm trong cột Ghi chú.</t>
         </is>
       </c>
-      <c r="E64" s="23" t="n"/>
-      <c r="F64" s="23" t="n"/>
-      <c r="G64" s="23" t="n"/>
-      <c r="H64" s="23" t="n"/>
-      <c r="I64" s="23" t="n"/>
+      <c r="E64" s="17" t="n"/>
+      <c r="F64" s="17" t="n"/>
+      <c r="G64" s="17" t="n"/>
+      <c r="H64" s="17" t="n"/>
+      <c r="I64" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -27411,18 +27483,18 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
+      <c r="B53" s="17" t="n"/>
+      <c r="C53" s="18" t="n"/>
       <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Dạng P01-sales: câu hỏi P01 hỏi bằng tài khoản sales. Mỗi câu được hỏi bằng cả 4 vai trò (manager, sales, production_a, it_admin).</t>
         </is>
       </c>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
+      <c r="E53" s="17" t="n"/>
+      <c r="F53" s="17" t="n"/>
+      <c r="G53" s="17" t="n"/>
+      <c r="H53" s="17" t="n"/>
+      <c r="I53" s="18" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="21" t="inlineStr">
@@ -27430,18 +27502,18 @@
           <t>Test Suite</t>
         </is>
       </c>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
+      <c r="B54" s="17" t="n"/>
+      <c r="C54" s="18" t="n"/>
       <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Nhóm (bộ) kiểm thử mà ca thuộc về.</t>
         </is>
       </c>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="17" t="n"/>
+      <c r="H54" s="17" t="n"/>
+      <c r="I54" s="18" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="21" t="inlineStr">
@@ -27449,18 +27521,18 @@
           <t>Tiêu đề (Title)</t>
         </is>
       </c>
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
+      <c r="B55" s="17" t="n"/>
+      <c r="C55" s="18" t="n"/>
       <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Tên ngắn của ca: câu hỏi chính được đem ra thử.</t>
         </is>
       </c>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="23" t="n"/>
-      <c r="H55" s="23" t="n"/>
-      <c r="I55" s="23" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="17" t="n"/>
+      <c r="G55" s="17" t="n"/>
+      <c r="H55" s="17" t="n"/>
+      <c r="I55" s="18" t="n"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="21" t="inlineStr">
@@ -27468,18 +27540,18 @@
           <t>Điều kiện tiên quyết (Pre-conditions)</t>
         </is>
       </c>
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
+      <c r="B56" s="17" t="n"/>
+      <c r="C56" s="18" t="n"/>
       <c r="D56" s="22" t="inlineStr">
         <is>
           <t>Cần có gì trước khi chạy: đăng nhập bằng vai trò nào, ngôn ngữ nào, hội thoại mới hay nhiều lượt trong cùng một hội thoại.</t>
         </is>
       </c>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="23" t="n"/>
-      <c r="H56" s="23" t="n"/>
-      <c r="I56" s="23" t="n"/>
+      <c r="E56" s="17" t="n"/>
+      <c r="F56" s="17" t="n"/>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="17" t="n"/>
+      <c r="I56" s="18" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="21" t="inlineStr">
@@ -27487,18 +27559,18 @@
           <t>Các bước (Test Steps)</t>
         </is>
       </c>
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="18" t="n"/>
       <c r="D57" s="22" t="inlineStr">
         <is>
           <t>Việc đã làm, theo thứ tự: gửi từng câu hỏi, rồi (nếu có) chạy một câu SQL độc lập trên kho dữ liệu để đối chiếu số.</t>
         </is>
       </c>
-      <c r="E57" s="23" t="n"/>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="23" t="n"/>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="n"/>
+      <c r="E57" s="17" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="17" t="n"/>
+      <c r="I57" s="18" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="21" t="inlineStr">
@@ -27506,18 +27578,18 @@
           <t>Dữ liệu kiểm thử (Test Data)</t>
         </is>
       </c>
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
+      <c r="B58" s="17" t="n"/>
+      <c r="C58" s="18" t="n"/>
       <c r="D58" s="22" t="inlineStr">
         <is>
           <t>Nguyên văn các câu hỏi đã gửi cho hệ thống.</t>
         </is>
       </c>
-      <c r="E58" s="23" t="n"/>
-      <c r="F58" s="23" t="n"/>
-      <c r="G58" s="23" t="n"/>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="23" t="n"/>
+      <c r="E58" s="17" t="n"/>
+      <c r="F58" s="17" t="n"/>
+      <c r="G58" s="17" t="n"/>
+      <c r="H58" s="17" t="n"/>
+      <c r="I58" s="18" t="n"/>
     </row>
     <row r="59" ht="32" customHeight="1">
       <c r="A59" s="21" t="inlineStr">
@@ -27525,18 +27597,18 @@
           <t>Kết quả mong đợi (Expected Result)</t>
         </is>
       </c>
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
+      <c r="B59" s="17" t="n"/>
+      <c r="C59" s="18" t="n"/>
       <c r="D59" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống phải làm để ca được coi là đạt: trạng thái cho phép (ok = có số liệu, needs_clarification = hỏi lại, denied = từ chối, no_data = không có dữ liệu), số dòng, loại biểu đồ, cụm chữ phải có hoặc không được có, và số có khớp kho dữ liệu hay không.</t>
         </is>
       </c>
-      <c r="E59" s="23" t="n"/>
-      <c r="F59" s="23" t="n"/>
-      <c r="G59" s="23" t="n"/>
-      <c r="H59" s="23" t="n"/>
-      <c r="I59" s="23" t="n"/>
+      <c r="E59" s="17" t="n"/>
+      <c r="F59" s="17" t="n"/>
+      <c r="G59" s="17" t="n"/>
+      <c r="H59" s="17" t="n"/>
+      <c r="I59" s="18" t="n"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="21" t="inlineStr">
@@ -27544,18 +27616,18 @@
           <t>Kết quả thực tế (Actual Result)</t>
         </is>
       </c>
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
+      <c r="B60" s="17" t="n"/>
+      <c r="C60" s="18" t="n"/>
       <c r="D60" s="22" t="inlineStr">
         <is>
           <t>Điều hệ thống đã trả về: trạng thái, câu trả lời nguyên văn (cắt ngắn), số dòng của bảng và loại biểu đồ.</t>
         </is>
       </c>
-      <c r="E60" s="23" t="n"/>
-      <c r="F60" s="23" t="n"/>
-      <c r="G60" s="23" t="n"/>
-      <c r="H60" s="23" t="n"/>
-      <c r="I60" s="23" t="n"/>
+      <c r="E60" s="17" t="n"/>
+      <c r="F60" s="17" t="n"/>
+      <c r="G60" s="17" t="n"/>
+      <c r="H60" s="17" t="n"/>
+      <c r="I60" s="18" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="21" t="inlineStr">
@@ -27563,18 +27635,18 @@
           <t>Trạng thái (Status)</t>
         </is>
       </c>
-      <c r="B61" s="23" t="n"/>
-      <c r="C61" s="23" t="n"/>
+      <c r="B61" s="17" t="n"/>
+      <c r="C61" s="18" t="n"/>
       <c r="D61" s="22" t="inlineStr">
         <is>
           <t>Passed = vai trò nhận đúng thứ được phép (có số liệu nếu được xem, bị từ chối nếu không được xem) và khi bị từ chối thì không có dòng dữ liệu nào lọt ra. Failed = có dữ liệu ngoài quyền hoặc trạng thái sai.</t>
         </is>
       </c>
-      <c r="E61" s="23" t="n"/>
-      <c r="F61" s="23" t="n"/>
-      <c r="G61" s="23" t="n"/>
-      <c r="H61" s="23" t="n"/>
-      <c r="I61" s="23" t="n"/>
+      <c r="E61" s="17" t="n"/>
+      <c r="F61" s="17" t="n"/>
+      <c r="G61" s="17" t="n"/>
+      <c r="H61" s="17" t="n"/>
+      <c r="I61" s="18" t="n"/>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="21" t="inlineStr">
@@ -27582,18 +27654,18 @@
           <t>Ý nghĩa của bộ này</t>
         </is>
       </c>
-      <c r="B62" s="23" t="n"/>
-      <c r="C62" s="23" t="n"/>
+      <c r="B62" s="17" t="n"/>
+      <c r="C62" s="18" t="n"/>
       <c r="D62" s="22" t="inlineStr">
         <is>
           <t>Chứng minh phân quyền do backend cưỡng chế trên cả đường truy vấn mẫu (Structured Intent) lẫn đường AI sinh SQL (RAG), kể cả với câu tấn công như bỏ qua hướng dẫn hoặc gõ thẳng SQL.</t>
         </is>
       </c>
-      <c r="E62" s="23" t="n"/>
-      <c r="F62" s="23" t="n"/>
-      <c r="G62" s="23" t="n"/>
-      <c r="H62" s="23" t="n"/>
-      <c r="I62" s="23" t="n"/>
+      <c r="E62" s="17" t="n"/>
+      <c r="F62" s="17" t="n"/>
+      <c r="G62" s="17" t="n"/>
+      <c r="H62" s="17" t="n"/>
+      <c r="I62" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -28629,15 +28701,15 @@
           <t>1. Cần bên độc lập</t>
         </is>
       </c>
-      <c r="B35" s="23" t="n"/>
+      <c r="B35" s="18" t="n"/>
       <c r="C35" s="22" t="inlineStr">
         <is>
           <t>Pentest chỉ có giá trị khi do người ngoài nhóm phát triển thực hiện, có phạm vi và ủy quyền bằng văn bản. Việc này cần chọn đơn vị, ký thỏa thuận và dành ngân sách; chưa nằm trong phạm vi của giai đoạn nguyên mẫu.</t>
         </is>
       </c>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
+      <c r="D35" s="17" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="18" t="n"/>
     </row>
     <row r="36" ht="62" customHeight="1">
       <c r="A36" s="21" t="inlineStr">
@@ -28645,15 +28717,15 @@
           <t>2. Cấu hình đang chạy sẽ không được dùng thật</t>
         </is>
       </c>
-      <c r="B36" s="23" t="n"/>
+      <c r="B36" s="18" t="n"/>
       <c r="C36" s="22" t="inlineStr">
         <is>
           <t>Bản demo đăng nhập bằng nút chọn vai trò, không mật khẩu, và chỉ có dữ liệu mẫu AdventureWorks. Pentest lúc này sẽ kiểm một cấu hình sẽ bị thay bằng xác thực thật, nên kết quả không dùng lại được.</t>
         </is>
       </c>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="18" t="n"/>
     </row>
     <row r="37" ht="62" customHeight="1">
       <c r="A37" s="21" t="inlineStr">
@@ -28661,15 +28733,15 @@
           <t>3. Hạ tầng dùng chung, miễn phí</t>
         </is>
       </c>
-      <c r="B37" s="23" t="n"/>
+      <c r="B37" s="18" t="n"/>
       <c r="C37" s="22" t="inlineStr">
         <is>
           <t>Demo chạy trên gói miễn phí của Vercel, Neon và các nhà cung cấp AI. Tấn công quy mô lớn có thể vi phạm điều khoản hoặc làm hết hạn mức dùng chung, nên chỉ chạy các kiểm tra nhẹ ở bảng trên.</t>
         </is>
       </c>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
+      <c r="D37" s="17" t="n"/>
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="18" t="n"/>
     </row>
     <row r="38" ht="62" customHeight="1">
       <c r="A38" s="21" t="inlineStr">
@@ -28677,15 +28749,15 @@
           <t>4. Đã xếp thành cổng bắt buộc</t>
         </is>
       </c>
-      <c r="B38" s="23" t="n"/>
+      <c r="B38" s="18" t="n"/>
       <c r="C38" s="22" t="inlineStr">
         <is>
           <t>Tài liệu giải pháp v1.1 (mục 11.2) và slide đều ghi: pentest độc lập hoàn tất là một điều kiện trước khi dùng dữ liệu thật.</t>
         </is>
       </c>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="18" t="n"/>
     </row>
     <row r="39" ht="62" customHeight="1">
       <c r="A39" s="21" t="inlineStr">
@@ -28693,15 +28765,15 @@
           <t>Bảng này chứng minh gì</t>
         </is>
       </c>
-      <c r="B39" s="23" t="n"/>
+      <c r="B39" s="18" t="n"/>
       <c r="C39" s="22" t="inlineStr">
         <is>
           <t>Trong các kịch bản đã thử từ bên ngoài, hệ thống từ chối truy cập không có hoặc sai token, không cho vượt quyền giữa các vai trò, không để người dùng xem kết quả hoặc hội thoại của người khác, và không lộ khóa, lời nhắc hay dữ liệu bảng mật khẩu khi bị chèn lệnh.</t>
         </is>
       </c>
-      <c r="D39" s="23" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="18" t="n"/>
     </row>
     <row r="40" ht="62" customHeight="1">
       <c r="A40" s="21" t="inlineStr">
@@ -28709,15 +28781,15 @@
           <t>Bảng này chưa chứng minh</t>
         </is>
       </c>
-      <c r="B40" s="23" t="n"/>
+      <c r="B40" s="18" t="n"/>
       <c r="C40" s="22" t="inlineStr">
         <is>
           <t>Không phải toàn bộ tấn công: chưa có quét lỗ hổng thư viện, kiểm tra cấu hình hạ tầng, kiểm tra mã nguồn, tấn công làm quá tải (DoS), thử đoán mật khẩu hay xác thực nhiều lớp (vì demo chưa dùng xác thực thật). Câu AI từ chối ở các ca chèn lệnh là hành vi quan sát được, không thay thế việc rà soát độc lập.</t>
         </is>
       </c>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
+      <c r="D40" s="17" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="18" t="n"/>
     </row>
     <row r="41" ht="62" customHeight="1">
       <c r="A41" s="21" t="inlineStr">
@@ -28725,15 +28797,15 @@
           <t>Phát hiện đã xử lý</t>
         </is>
       </c>
-      <c r="B41" s="23" t="n"/>
+      <c r="B41" s="18" t="n"/>
       <c r="C41" s="22" t="inlineStr">
         <is>
           <t>Ca S42 ban đầu không đạt: trang chủ thiếu tiêu đề X-Content-Type-Options và X-Frame-Options (chống nhúng khung). Đã thêm vào vercel.json và triển khai lại; kết quả trong bảng là sau khi sửa nếu ghi Đạt.</t>
         </is>
       </c>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
+      <c r="D41" s="17" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -28991,10 +29063,10 @@
           <t>Các mục tiêu chất lượng trong tài liệu giải pháp: chính xác, bảo mật, truy vết, dễ dùng, hiệu năng.</t>
         </is>
       </c>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="23" t="n"/>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="23" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="18" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
@@ -29007,10 +29079,10 @@
           <t>Việc làm để chứng minh yêu cầu được đáp ứng.</t>
         </is>
       </c>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="23" t="n"/>
-      <c r="E12" s="23" t="n"/>
-      <c r="F12" s="23" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="18" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
@@ -29023,10 +29095,10 @@
           <t>Bộ kiểm thử liên quan, số ca và số ca đạt (tính bằng công thức từ các sheet chi tiết). Ô trống nghĩa là yêu cầu đó chưa có ca kiểm thử riêng.</t>
         </is>
       </c>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="23" t="n"/>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="23" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="18" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
@@ -29039,10 +29111,10 @@
           <t>Chỗ còn thiếu hoặc điều cần lưu ý khi đọc kết quả.</t>
         </is>
       </c>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="23" t="n"/>
-      <c r="E14" s="23" t="n"/>
-      <c r="F14" s="23" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -36759,18 +36831,18 @@
           <t>Đối chiếu độc lập là gì</t>
         </is>
       </c>
-      <c r="B169" s="23" t="n"/>
-      <c r="C169" s="23" t="n"/>
+      <c r="B169" s="17" t="n"/>
+      <c r="C169" s="18" t="n"/>
       <c r="D169" s="22" t="inlineStr">
         <is>
           <t>Với mỗi câu trả lời có bảng số liệu, một đoạn mã riêng tính lại các con số bằng câu SQL viết tay, chạy trực tiếp trên kho dữ liệu bằng tài khoản chỉ đọc, không dùng bộ dựng truy vấn của ứng dụng, rồi so từng giá trị. Hai đường độc lập cho cùng một số thì kết quả đáng tin.</t>
         </is>
       </c>
-      <c r="E169" s="23" t="n"/>
-      <c r="F169" s="23" t="n"/>
-      <c r="G169" s="23" t="n"/>
-      <c r="H169" s="23" t="n"/>
-      <c r="I169" s="23" t="n"/>
+      <c r="E169" s="17" t="n"/>
+      <c r="F169" s="17" t="n"/>
+      <c r="G169" s="17" t="n"/>
+      <c r="H169" s="17" t="n"/>
+      <c r="I169" s="18" t="n"/>
     </row>
     <row r="170" ht="32" customHeight="1">
       <c r="A170" s="21" t="inlineStr">
@@ -36778,18 +36850,18 @@
           <t>Kết quả đối chiếu</t>
         </is>
       </c>
-      <c r="B170" s="23" t="n"/>
-      <c r="C170" s="23" t="n"/>
+      <c r="B170" s="17" t="n"/>
+      <c r="C170" s="18" t="n"/>
       <c r="D170" s="22" t="inlineStr">
         <is>
           <t>Khớp = mọi giá trị đã so đều bằng nhau (sai số tối đa 0,01 cho tiền và sản lượng; 0,000001 cho tỷ lệ). Lệch = có giá trị khác. Chưa đối chiếu = chưa có truy vấn độc lập cho kiểu kết quả đó (ví dụ theo sản phẩm, ngành hàng, dây chuyền, lý do phế phẩm, tăng trưởng); lý do ghi ở cột Ghi chú.</t>
         </is>
       </c>
-      <c r="E170" s="23" t="n"/>
-      <c r="F170" s="23" t="n"/>
-      <c r="G170" s="23" t="n"/>
-      <c r="H170" s="23" t="n"/>
-      <c r="I170" s="23" t="n"/>
+      <c r="E170" s="17" t="n"/>
+      <c r="F170" s="17" t="n"/>
+      <c r="G170" s="17" t="n"/>
+      <c r="H170" s="17" t="n"/>
+      <c r="I170" s="18" t="n"/>
     </row>
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="21" t="inlineStr">
@@ -36797,18 +36869,18 @@
           <t>Phạm vi</t>
         </is>
       </c>
-      <c r="B171" s="23" t="n"/>
-      <c r="C171" s="23" t="n"/>
+      <c r="B171" s="17" t="n"/>
+      <c r="C171" s="18" t="n"/>
       <c r="D171" s="22" t="inlineStr">
         <is>
           <t>chính = câu trả lời chính; tên phần = một phần của tin nhắn nhiều yêu cầu.</t>
         </is>
       </c>
-      <c r="E171" s="23" t="n"/>
-      <c r="F171" s="23" t="n"/>
-      <c r="G171" s="23" t="n"/>
-      <c r="H171" s="23" t="n"/>
-      <c r="I171" s="23" t="n"/>
+      <c r="E171" s="17" t="n"/>
+      <c r="F171" s="17" t="n"/>
+      <c r="G171" s="17" t="n"/>
+      <c r="H171" s="17" t="n"/>
+      <c r="I171" s="18" t="n"/>
     </row>
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="21" t="inlineStr">
@@ -36816,18 +36888,18 @@
           <t>Số giá trị đã so / lệch</t>
         </is>
       </c>
-      <c r="B172" s="23" t="n"/>
-      <c r="C172" s="23" t="n"/>
+      <c r="B172" s="17" t="n"/>
+      <c r="C172" s="18" t="n"/>
       <c r="D172" s="22" t="inlineStr">
         <is>
           <t>Số ô số liệu được so với kho dữ liệu và số ô khác nhau.</t>
         </is>
       </c>
-      <c r="E172" s="23" t="n"/>
-      <c r="F172" s="23" t="n"/>
-      <c r="G172" s="23" t="n"/>
-      <c r="H172" s="23" t="n"/>
-      <c r="I172" s="23" t="n"/>
+      <c r="E172" s="17" t="n"/>
+      <c r="F172" s="17" t="n"/>
+      <c r="G172" s="17" t="n"/>
+      <c r="H172" s="17" t="n"/>
+      <c r="I172" s="18" t="n"/>
     </row>
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="21" t="inlineStr">
@@ -36835,30 +36907,30 @@
           <t>Dự báo</t>
         </is>
       </c>
-      <c r="B173" s="23" t="n"/>
-      <c r="C173" s="23" t="n"/>
+      <c r="B173" s="17" t="n"/>
+      <c r="C173" s="18" t="n"/>
       <c r="D173" s="22" t="inlineStr">
         <is>
           <t>Chỉ so phần số liệu đã ghi nhận trong biểu đồ; giá trị dự báo được kiểm bằng kiểm thử tự động so với thư viện statsmodels.</t>
         </is>
       </c>
-      <c r="E173" s="23" t="n"/>
-      <c r="F173" s="23" t="n"/>
-      <c r="G173" s="23" t="n"/>
-      <c r="H173" s="23" t="n"/>
-      <c r="I173" s="23" t="n"/>
+      <c r="E173" s="17" t="n"/>
+      <c r="F173" s="17" t="n"/>
+      <c r="G173" s="17" t="n"/>
+      <c r="H173" s="17" t="n"/>
+      <c r="I173" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D173:I173"/>
+    <mergeCell ref="D172:I172"/>
     <mergeCell ref="D170:I170"/>
-    <mergeCell ref="D172:I172"/>
-    <mergeCell ref="D173:I173"/>
     <mergeCell ref="A169:C169"/>
     <mergeCell ref="A170:C170"/>
-    <mergeCell ref="A172:C172"/>
     <mergeCell ref="D169:I169"/>
     <mergeCell ref="A173:C173"/>
     <mergeCell ref="D171:I171"/>
+    <mergeCell ref="A172:C172"/>
     <mergeCell ref="A171:C171"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record the off-topic cost limit in the Excel, the script and the limits note
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -1856,6 +1856,13 @@
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
+          <t>• Câu hỏi ngoài chủ đề (bài tập, viết văn, viết code, dịch): hệ thống từ chối nhưng mỗi câu vẫn tốn 1 đến 2 lần gọi AI, và có dịch văn bản ngắn; chưa có giới hạn số câu theo từng người dùng. Thử 6 câu trên bản demo ngày 17/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
           <t>• Hiệu năng và độ ổn định của AI bị chi phối bởi quota gói miễn phí; con số chốt cần đo lại với gói trả phí.</t>
         </is>
       </c>
@@ -2229,7 +2236,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="35">
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B54:I54"/>
     <mergeCell ref="A66:I66"/>
@@ -2260,6 +2267,7 @@
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="B55:I55"/>
     <mergeCell ref="B6:I6"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="A45:I45"/>
     <mergeCell ref="B5:I5"/>

</xml_diff>

<commit_message>
Voice input is on in the hosted demo (Groq Whisper); update the Excel, script and slides
</commit_message>
<xml_diff>
--- a/docs/ACBI_bao_cao_kiem_thu.xlsx
+++ b/docs/ACBI_bao_cao_kiem_thu.xlsx
@@ -4491,14 +4491,14 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Chưa bật (không có khóa Groq trên Vercel)</t>
+          <t>Bật từ 17/10/2026 (Groq Whisper); đã thử bằng một file âm thanh tiếng Anh, chưa thử tiếng Việt</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Nhà cung cấp AI đang dùng: Gemini và LiteRouter (bản demo), Groq tùy chọn, Ollama chạy trên máy nội bộ (không ra ngoài).</t>
+          <t>Nhà cung cấp AI đang dùng: Gemini và LiteRouter (bản demo); Groq chỉ dùng để chuyển giọng nói (Whisper), không dùng để hiểu câu hỏi; Ollama chạy trên máy nội bộ (không ra ngoài).</t>
         </is>
       </c>
     </row>

</xml_diff>